<commit_message>
Add usage instructions to top of both Excel sheets
- Sheet 1 'Synthetic Notes': Added navigation guide explaining blue/green/gold
  color coding, how to scroll through 68 columns, and keyboard shortcuts
- Sheet 2 'Answer Key': Added step-by-step guide for how to verify a system's
  output against ground truth, plus expanded color legend with all grade levels
</commit_message>
<xml_diff>
--- a/data/synthetic_notes.xlsx
+++ b/data/synthetic_notes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Answer Key" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthetic Notes'!$A$1:$BP$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthetic Notes'!$A$16:$BP$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,13 +20,34 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5496"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002F5496"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -38,12 +59,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="002F5496"/>
-      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -60,16 +75,14 @@
       <i val="1"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002F5496"/>
-      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -78,8 +91,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
-        <bgColor rgb="002F5496"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -98,6 +111,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFC000"/>
         <bgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
       </patternFill>
     </fill>
     <fill>
@@ -136,8 +155,14 @@
         <bgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -151,13 +176,42 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,40 +223,42 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -568,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP4"/>
+  <dimension ref="A1:BP19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -644,397 +700,515 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>📋 SYNTHETIC NOTES — HOW TO USE THIS SHEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WHAT IS THIS?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>This sheet contains 3 synthetic clinical notes for Sickle Cell Disease patients, formatted in the same</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>68-column structure as clincal_notes.csv. Each note has known ground-truth SCOGS grades for testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO NAVIGATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>• Columns A–O (blue) = Patient demographics &amp; clinical note text. Column K has the full note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>• Columns P–BP (green) = The 53 SCOGS outcome columns. Empty = outcome is absent from the note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>• Gold-highlighted cells = Outcomes that ARE present, with the SCOGS grade (1–5) as the value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>• Scroll RIGHT to see all 53 outcome columns. Use Ctrl+Right Arrow to jump to the next graded cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>• The header row (row 16) is frozen — it stays visible as you scroll down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>COLOR KEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Blue = Demographics</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Green = Outcome (absent)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>Gold = Outcome (graded)</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
           <t>patient_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>visit_datetime</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>facility_type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>pain_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>pain_intensity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>admitted</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>hemoglobin</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>oxygen_saturation</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J16" s="9" t="inlineStr">
         <is>
           <t>weather</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K16" s="9" t="inlineStr">
         <is>
           <t>clinical_note</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>dob</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M16" s="9" t="inlineStr">
         <is>
           <t>diagnosis_date</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N16" s="9" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O16" s="9" t="inlineStr">
         <is>
           <t>race</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P16" s="9" t="inlineStr">
         <is>
           <t>arrhythmia</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>deep_vein_thrombosis_dvt</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R16" s="9" t="inlineStr">
         <is>
           <t>diastolic_dysfunction</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S16" s="9" t="inlineStr">
         <is>
           <t>heart_failure_exacerbation</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T16" s="9" t="inlineStr">
         <is>
           <t>myocardial_infarction</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U16" s="9" t="inlineStr">
         <is>
           <t>systemic_arterial_hypertension</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V16" s="9" t="inlineStr">
         <is>
           <t>systolic_dysfunction</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W16" s="9" t="inlineStr">
         <is>
           <t>tricuspid_regurgitant_jet_velocity_trv_elevation_on_echocardiogram</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X16" s="9" t="inlineStr">
         <is>
           <t>cerebral_vasculopathy</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y16" s="9" t="inlineStr">
         <is>
           <t>chronic_pain</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z16" s="9" t="inlineStr">
         <is>
           <t>cognitive_dysfunction</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA16" s="9" t="inlineStr">
         <is>
           <t>elevated_transcranial_doppler_tcd_ultrasonography_velocity</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB16" s="9" t="inlineStr">
         <is>
           <t>posterior_reversible_encephalopathy_syndrome_pres</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC16" s="9" t="inlineStr">
         <is>
           <t>silent_cerebral_infarct</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD16" s="9" t="inlineStr">
         <is>
           <t>stroke_hemorrhagic_or_ischemic</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE16" s="9" t="inlineStr">
         <is>
           <t>hearing_loss_in_at_least_one_ear</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF16" s="9" t="inlineStr">
         <is>
           <t>sickle_cell_retinopathy_scr</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG16" s="9" t="inlineStr">
         <is>
           <t>cholecystitis_cholelithiasis_gallstones</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH16" s="9" t="inlineStr">
         <is>
           <t>acute_kidney_injury_aki</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI16" s="9" t="inlineStr">
         <is>
           <t>acute_papillary_necrosis</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ16" s="9" t="inlineStr">
         <is>
           <t>chronic_kidney_disease_ckd</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK16" s="9" t="inlineStr">
         <is>
           <t>female_ovarian_dysfunction</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL16" s="9" t="inlineStr">
         <is>
           <t>male_impairments</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM16" s="9" t="inlineStr">
         <is>
           <t>priapism</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN16" s="9" t="inlineStr">
         <is>
           <t>delayed_puberty</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO16" s="9" t="inlineStr">
         <is>
           <t>malnutrition_leading_to_stunting_decreased_height_velocity</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP16" s="9" t="inlineStr">
         <is>
           <t>underweight</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ16" s="9" t="inlineStr">
         <is>
           <t>acute_sickle_cell_pain_episode</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR16" s="9" t="inlineStr">
         <is>
           <t>acute_splenic_sequestration</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS16" s="9" t="inlineStr">
         <is>
           <t>alloimmunization_delayed_hemolytic_transfusion_reaction_dhtr</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT16" s="9" t="inlineStr">
         <is>
           <t>chronic_hypersplenism</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU16" s="9" t="inlineStr">
         <is>
           <t>hepatopathy</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV16" s="9" t="inlineStr">
         <is>
           <t>splenic_infarction</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW16" s="9" t="inlineStr">
         <is>
           <t>transfusional_iron_overload_hemochromatosis_or_hemosiderosis</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX16" s="9" t="inlineStr">
         <is>
           <t>transient_aplastic_crisis_secondary_to_parvovirus_b19_infection</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY16" s="9" t="inlineStr">
         <is>
           <t>fever</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ16" s="9" t="inlineStr">
         <is>
           <t>sepsis</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA16" s="9" t="inlineStr">
         <is>
           <t>malignant_neoplasms</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB16" s="9" t="inlineStr">
         <is>
           <t>avascular_necrosis_of_joints_avn</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC16" s="9" t="inlineStr">
         <is>
           <t>leg_ulcer</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD16" s="9" t="inlineStr">
         <is>
           <t>osteomyelitis</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE16" s="9" t="inlineStr">
         <is>
           <t>osteoporosis</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF16" s="9" t="inlineStr">
         <is>
           <t>acute_multiorgan_failure</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BG16" s="9" t="inlineStr">
         <is>
           <t>fetal_growth_restriction</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BH16" s="9" t="inlineStr">
         <is>
           <t>pregnancy_loss</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BI16" s="9" t="inlineStr">
         <is>
           <t>premature_delivery</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BJ16" s="9" t="inlineStr">
         <is>
           <t>depression</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BK16" s="9" t="inlineStr">
         <is>
           <t>acute_chest_syndrome_acs</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BL16" s="9" t="inlineStr">
         <is>
           <t>asthma_exacerbation</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BM16" s="9" t="inlineStr">
         <is>
           <t>chronic_restrictive_lung_physiology</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BN16" s="9" t="inlineStr">
         <is>
           <t>pulmonary_embolism_pe</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BO16" s="9" t="inlineStr">
         <is>
           <t>pulmonary_hypertension</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BP16" s="9" t="inlineStr">
         <is>
           <t>sleep_apnea_obstructive_or_central</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="200" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="17" ht="200" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>SYNTH_001</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>3/15/25</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>ER</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Leg Pain</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>Memphis</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>7.8</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J17" s="10" t="inlineStr">
         <is>
           <t>Warm</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K17" s="11" t="inlineStr">
         <is>
           <t>SUBJECTIVE: 22-year-old female with known sickle cell disease (HbSS), diagnosed at age 2, presents to the emergency department with bilateral lower extremity pain that began approximately 6 hours ago. She describes the pain as deep, aching, and throbbing, rated 7 out of 10 in intensity. She reports taking ibuprofen 600 mg and acetaminophen 1000 mg at home without adequate relief. She also notes feeling warm and mildly fatigued. She denies cough, shortness of breath, chest pain, abdominal pain, headache, vision changes, or urinary symptoms. No recent travel or sick contacts. No history of DVT or pulmonary embolism.
 OBJECTIVE: Temperature 38.3 degrees Celsius (101.0 degrees Fahrenheit), heart rate 98 bpm, blood pressure 112/68 mmHg, respiratory rate 18 breaths/min, SpO2 98% on room air. General: Alert, oriented, appears uncomfortable but not in acute distress. HEENT: Scleral icterus noted bilaterally. Lungs: Clear to auscultation bilaterally, no wheezes, crackles, or rhonchi. Cardiovascular: Regular rate and rhythm, no murmurs, rubs, or gallops. Abdomen: Soft, non-tender, non-distended, no hepatosplenomegaly. Extremities: Bilateral tibial tenderness to palpation without swelling or erythema, no edema, no calf tenderness, no leg ulcers. Neurological: Alert and oriented x4, cranial nerves II-XII intact, no focal motor or sensory deficits, gait not assessed due to pain.
@@ -1042,140 +1216,140 @@
 ASSESSMENT AND PLAN: (1) Acute sickle cell vaso-occlusive pain episode. Administered IV normal saline bolus 1 liter, IV morphine 4 mg with adequate pain relief achieved (pain reduced to 3/10). Patient monitored in ED for 4 hours with improvement. Not admitted. Discharged home with oral oxycodone 5 mg every 4-6 hours as needed for pain, ibuprofen 600 mg every 8 hours, and instructions to return if fever exceeds 38.5 degrees Celsius, or if she develops chest pain, shortness of breath, or worsening symptoms. Follow-up with hematology clinic in 48 hours. (2) Low-grade fever, temperature 38.3 degrees Celsius. Most likely related to vaso-occlusive crisis. Blood cultures pending. No signs of acute chest syndrome, sepsis, or other infectious source identified.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L17" s="10" t="inlineStr">
         <is>
           <t>4/10/03</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="M17" s="10" t="inlineStr">
         <is>
           <t>6/20/05</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="N17" s="10" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O17" s="10" t="inlineStr">
         <is>
           <t>Black or African American</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr"/>
-      <c r="Q2" s="4" t="inlineStr"/>
-      <c r="R2" s="4" t="inlineStr"/>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
-      <c r="V2" s="4" t="inlineStr"/>
-      <c r="W2" s="4" t="inlineStr"/>
-      <c r="X2" s="4" t="inlineStr"/>
-      <c r="Y2" s="4" t="inlineStr"/>
-      <c r="Z2" s="4" t="inlineStr"/>
-      <c r="AA2" s="4" t="inlineStr"/>
-      <c r="AB2" s="4" t="inlineStr"/>
-      <c r="AC2" s="4" t="inlineStr"/>
-      <c r="AD2" s="4" t="inlineStr"/>
-      <c r="AE2" s="4" t="inlineStr"/>
-      <c r="AF2" s="4" t="inlineStr"/>
-      <c r="AG2" s="4" t="inlineStr"/>
-      <c r="AH2" s="4" t="inlineStr"/>
-      <c r="AI2" s="4" t="inlineStr"/>
-      <c r="AJ2" s="4" t="inlineStr"/>
-      <c r="AK2" s="4" t="inlineStr"/>
-      <c r="AL2" s="4" t="inlineStr"/>
-      <c r="AM2" s="4" t="inlineStr"/>
-      <c r="AN2" s="4" t="inlineStr"/>
-      <c r="AO2" s="4" t="inlineStr"/>
-      <c r="AP2" s="4" t="inlineStr"/>
-      <c r="AQ2" s="5" t="inlineStr">
+      <c r="P17" s="12" t="inlineStr"/>
+      <c r="Q17" s="12" t="inlineStr"/>
+      <c r="R17" s="12" t="inlineStr"/>
+      <c r="S17" s="12" t="inlineStr"/>
+      <c r="T17" s="12" t="inlineStr"/>
+      <c r="U17" s="12" t="inlineStr"/>
+      <c r="V17" s="12" t="inlineStr"/>
+      <c r="W17" s="12" t="inlineStr"/>
+      <c r="X17" s="12" t="inlineStr"/>
+      <c r="Y17" s="12" t="inlineStr"/>
+      <c r="Z17" s="12" t="inlineStr"/>
+      <c r="AA17" s="12" t="inlineStr"/>
+      <c r="AB17" s="12" t="inlineStr"/>
+      <c r="AC17" s="12" t="inlineStr"/>
+      <c r="AD17" s="12" t="inlineStr"/>
+      <c r="AE17" s="12" t="inlineStr"/>
+      <c r="AF17" s="12" t="inlineStr"/>
+      <c r="AG17" s="12" t="inlineStr"/>
+      <c r="AH17" s="12" t="inlineStr"/>
+      <c r="AI17" s="12" t="inlineStr"/>
+      <c r="AJ17" s="12" t="inlineStr"/>
+      <c r="AK17" s="12" t="inlineStr"/>
+      <c r="AL17" s="12" t="inlineStr"/>
+      <c r="AM17" s="12" t="inlineStr"/>
+      <c r="AN17" s="12" t="inlineStr"/>
+      <c r="AO17" s="12" t="inlineStr"/>
+      <c r="AP17" s="12" t="inlineStr"/>
+      <c r="AQ17" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AR2" s="4" t="inlineStr"/>
-      <c r="AS2" s="4" t="inlineStr"/>
-      <c r="AT2" s="4" t="inlineStr"/>
-      <c r="AU2" s="4" t="inlineStr"/>
-      <c r="AV2" s="4" t="inlineStr"/>
-      <c r="AW2" s="4" t="inlineStr"/>
-      <c r="AX2" s="4" t="inlineStr"/>
-      <c r="AY2" s="5" t="inlineStr">
+      <c r="AR17" s="12" t="inlineStr"/>
+      <c r="AS17" s="12" t="inlineStr"/>
+      <c r="AT17" s="12" t="inlineStr"/>
+      <c r="AU17" s="12" t="inlineStr"/>
+      <c r="AV17" s="12" t="inlineStr"/>
+      <c r="AW17" s="12" t="inlineStr"/>
+      <c r="AX17" s="12" t="inlineStr"/>
+      <c r="AY17" s="13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AZ2" s="4" t="inlineStr"/>
-      <c r="BA2" s="4" t="inlineStr"/>
-      <c r="BB2" s="4" t="inlineStr"/>
-      <c r="BC2" s="4" t="inlineStr"/>
-      <c r="BD2" s="4" t="inlineStr"/>
-      <c r="BE2" s="4" t="inlineStr"/>
-      <c r="BF2" s="4" t="inlineStr"/>
-      <c r="BG2" s="4" t="inlineStr"/>
-      <c r="BH2" s="4" t="inlineStr"/>
-      <c r="BI2" s="4" t="inlineStr"/>
-      <c r="BJ2" s="4" t="inlineStr"/>
-      <c r="BK2" s="4" t="inlineStr"/>
-      <c r="BL2" s="4" t="inlineStr"/>
-      <c r="BM2" s="4" t="inlineStr"/>
-      <c r="BN2" s="4" t="inlineStr"/>
-      <c r="BO2" s="4" t="inlineStr"/>
-      <c r="BP2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3" ht="200" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="AZ17" s="12" t="inlineStr"/>
+      <c r="BA17" s="12" t="inlineStr"/>
+      <c r="BB17" s="12" t="inlineStr"/>
+      <c r="BC17" s="12" t="inlineStr"/>
+      <c r="BD17" s="12" t="inlineStr"/>
+      <c r="BE17" s="12" t="inlineStr"/>
+      <c r="BF17" s="12" t="inlineStr"/>
+      <c r="BG17" s="12" t="inlineStr"/>
+      <c r="BH17" s="12" t="inlineStr"/>
+      <c r="BI17" s="12" t="inlineStr"/>
+      <c r="BJ17" s="12" t="inlineStr"/>
+      <c r="BK17" s="12" t="inlineStr"/>
+      <c r="BL17" s="12" t="inlineStr"/>
+      <c r="BM17" s="12" t="inlineStr"/>
+      <c r="BN17" s="12" t="inlineStr"/>
+      <c r="BO17" s="12" t="inlineStr"/>
+      <c r="BP17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18" ht="200" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>SYNTH_002</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>7/22/25</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>ER</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Chest Pain</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Memphis</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>88</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>Hot</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>SUBJECTIVE: 17-year-old male with sickle cell disease (HbSS), on chronic transfusion program, presents with acute onset of severe generalized body pain rated 9 out of 10, productive cough with yellowish sputum, and progressive shortness of breath over the past 18 hours. He reports fever at home measured at 39.2 degrees Celsius (102.6 degrees Fahrenheit). He has had three prior hospitalizations for acute chest syndrome in the past two years. He denies headache, visual changes, abdominal pain, dysuria, or hematuria. No history of leg swelling, DVT, or pulmonary embolism. No depressive symptoms reported.
 OBJECTIVE: Temperature 39.2 degrees Celsius (102.6 degrees Fahrenheit), heart rate 118 bpm, blood pressure 102/58 mmHg, respiratory rate 28 breaths/min, SpO2 88% on room air. General: Acutely ill-appearing, diaphoretic, using accessory muscles of respiration. HEENT: Scleral icterus, dry mucous membranes. Lungs: Decreased breath sounds at right lower lobe with dullness to percussion and bronchial breath sounds; scattered crackles bilaterally. Cardiovascular: Tachycardic, regular rhythm, grade II/VI systolic flow murmur at left sternal border. Abdomen: Mild splenomegaly palpated 2 cm below left costal margin, no acute tenderness. Extremities: Diffuse tenderness in bilateral upper and lower extremities, no edema, no calf tenderness, no leg ulcers. Neurological: Alert and oriented x3, no focal neurological deficits, moving all extremities symmetrically, cranial nerves intact.
@@ -1185,144 +1359,144 @@
 DISCHARGE DIAGNOSES: (1) Acute chest syndrome, severe, requiring high-flow oxygen therapy and exchange transfusion. (2) Acute sickle cell vaso-occlusive pain crisis complicated by acute chest syndrome. (3) Fever secondary to acute chest syndrome.</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L18" s="10" t="inlineStr">
         <is>
           <t>11/3/07</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="M18" s="10" t="inlineStr">
         <is>
           <t>2/15/08</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="N18" s="10" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O18" s="10" t="inlineStr">
         <is>
           <t>Black or African American</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr"/>
-      <c r="Q3" s="4" t="inlineStr"/>
-      <c r="R3" s="4" t="inlineStr"/>
-      <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
-      <c r="V3" s="4" t="inlineStr"/>
-      <c r="W3" s="4" t="inlineStr"/>
-      <c r="X3" s="4" t="inlineStr"/>
-      <c r="Y3" s="4" t="inlineStr"/>
-      <c r="Z3" s="4" t="inlineStr"/>
-      <c r="AA3" s="4" t="inlineStr"/>
-      <c r="AB3" s="4" t="inlineStr"/>
-      <c r="AC3" s="4" t="inlineStr"/>
-      <c r="AD3" s="4" t="inlineStr"/>
-      <c r="AE3" s="4" t="inlineStr"/>
-      <c r="AF3" s="4" t="inlineStr"/>
-      <c r="AG3" s="4" t="inlineStr"/>
-      <c r="AH3" s="4" t="inlineStr"/>
-      <c r="AI3" s="4" t="inlineStr"/>
-      <c r="AJ3" s="4" t="inlineStr"/>
-      <c r="AK3" s="4" t="inlineStr"/>
-      <c r="AL3" s="4" t="inlineStr"/>
-      <c r="AM3" s="4" t="inlineStr"/>
-      <c r="AN3" s="4" t="inlineStr"/>
-      <c r="AO3" s="4" t="inlineStr"/>
-      <c r="AP3" s="4" t="inlineStr"/>
-      <c r="AQ3" s="5" t="inlineStr">
+      <c r="P18" s="12" t="inlineStr"/>
+      <c r="Q18" s="12" t="inlineStr"/>
+      <c r="R18" s="12" t="inlineStr"/>
+      <c r="S18" s="12" t="inlineStr"/>
+      <c r="T18" s="12" t="inlineStr"/>
+      <c r="U18" s="12" t="inlineStr"/>
+      <c r="V18" s="12" t="inlineStr"/>
+      <c r="W18" s="12" t="inlineStr"/>
+      <c r="X18" s="12" t="inlineStr"/>
+      <c r="Y18" s="12" t="inlineStr"/>
+      <c r="Z18" s="12" t="inlineStr"/>
+      <c r="AA18" s="12" t="inlineStr"/>
+      <c r="AB18" s="12" t="inlineStr"/>
+      <c r="AC18" s="12" t="inlineStr"/>
+      <c r="AD18" s="12" t="inlineStr"/>
+      <c r="AE18" s="12" t="inlineStr"/>
+      <c r="AF18" s="12" t="inlineStr"/>
+      <c r="AG18" s="12" t="inlineStr"/>
+      <c r="AH18" s="12" t="inlineStr"/>
+      <c r="AI18" s="12" t="inlineStr"/>
+      <c r="AJ18" s="12" t="inlineStr"/>
+      <c r="AK18" s="12" t="inlineStr"/>
+      <c r="AL18" s="12" t="inlineStr"/>
+      <c r="AM18" s="12" t="inlineStr"/>
+      <c r="AN18" s="12" t="inlineStr"/>
+      <c r="AO18" s="12" t="inlineStr"/>
+      <c r="AP18" s="12" t="inlineStr"/>
+      <c r="AQ18" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AR3" s="4" t="inlineStr"/>
-      <c r="AS3" s="4" t="inlineStr"/>
-      <c r="AT3" s="4" t="inlineStr"/>
-      <c r="AU3" s="4" t="inlineStr"/>
-      <c r="AV3" s="4" t="inlineStr"/>
-      <c r="AW3" s="4" t="inlineStr"/>
-      <c r="AX3" s="4" t="inlineStr"/>
-      <c r="AY3" s="5" t="inlineStr">
+      <c r="AR18" s="12" t="inlineStr"/>
+      <c r="AS18" s="12" t="inlineStr"/>
+      <c r="AT18" s="12" t="inlineStr"/>
+      <c r="AU18" s="12" t="inlineStr"/>
+      <c r="AV18" s="12" t="inlineStr"/>
+      <c r="AW18" s="12" t="inlineStr"/>
+      <c r="AX18" s="12" t="inlineStr"/>
+      <c r="AY18" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AZ3" s="4" t="inlineStr"/>
-      <c r="BA3" s="4" t="inlineStr"/>
-      <c r="BB3" s="4" t="inlineStr"/>
-      <c r="BC3" s="4" t="inlineStr"/>
-      <c r="BD3" s="4" t="inlineStr"/>
-      <c r="BE3" s="4" t="inlineStr"/>
-      <c r="BF3" s="4" t="inlineStr"/>
-      <c r="BG3" s="4" t="inlineStr"/>
-      <c r="BH3" s="4" t="inlineStr"/>
-      <c r="BI3" s="4" t="inlineStr"/>
-      <c r="BJ3" s="4" t="inlineStr"/>
-      <c r="BK3" s="5" t="inlineStr">
+      <c r="AZ18" s="12" t="inlineStr"/>
+      <c r="BA18" s="12" t="inlineStr"/>
+      <c r="BB18" s="12" t="inlineStr"/>
+      <c r="BC18" s="12" t="inlineStr"/>
+      <c r="BD18" s="12" t="inlineStr"/>
+      <c r="BE18" s="12" t="inlineStr"/>
+      <c r="BF18" s="12" t="inlineStr"/>
+      <c r="BG18" s="12" t="inlineStr"/>
+      <c r="BH18" s="12" t="inlineStr"/>
+      <c r="BI18" s="12" t="inlineStr"/>
+      <c r="BJ18" s="12" t="inlineStr"/>
+      <c r="BK18" s="13" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="BL3" s="4" t="inlineStr"/>
-      <c r="BM3" s="4" t="inlineStr"/>
-      <c r="BN3" s="4" t="inlineStr"/>
-      <c r="BO3" s="4" t="inlineStr"/>
-      <c r="BP3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4" ht="200" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="BL18" s="12" t="inlineStr"/>
+      <c r="BM18" s="12" t="inlineStr"/>
+      <c r="BN18" s="12" t="inlineStr"/>
+      <c r="BO18" s="12" t="inlineStr"/>
+      <c r="BP18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19" ht="200" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>SYNTH_003</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>1/8/26</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>ER</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Chest Pain</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>Memphis</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>79</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J19" s="10" t="inlineStr">
         <is>
           <t>Cold</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>SUBJECTIVE: 29-year-old male with sickle cell disease (HbSC), known history of avascular necrosis of the right hip (managed conservatively), presents via EMS to the emergency department with acute severe chest pain, progressive dyspnea, and high-grade fever for the past 8 hours. His wife reports he had been experiencing a vaso-occlusive pain crisis at home for two days managed with oral hydromorphone, but acutely worsened with onset of chest pain and difficulty breathing. She notes he became confused and less responsive during transport. No prior history of stroke, DVT, or PE. No psychiatric history or depressive symptoms.
 OBJECTIVE: Temperature 39.8 degrees Celsius (103.6 degrees Fahrenheit), heart rate 132 bpm, blood pressure 78/42 mmHg, respiratory rate 36 breaths/min, SpO2 79% on 15 L non-rebreather mask. General: Critically ill-appearing, obtunded, diaphoretic, severe respiratory distress with use of accessory muscles, intercostal and suprasternal retractions. HEENT: Scleral icterus, dry mucous membranes. Lungs: Diffuse bilateral crackles with diminished breath sounds in bilateral lower lobes. Cardiovascular: Tachycardic, distant heart sounds, no appreciable murmur. Abdomen: Distended, diffusely tender, hepatomegaly palpated 4 cm below right costal margin. Extremities: Cool, mottled, capillary refill greater than 4 seconds bilaterally, no peripheral edema, no leg ulcers. Neurological: GCS 10 (E2 V3 M5), pupils 3 mm bilaterally and reactive, withdraws to pain in all extremities. No lateralizing signs.
@@ -1333,98 +1507,114 @@
 DISCHARGE DIAGNOSES: (1) Acute chest syndrome, life-threatening, requiring invasive mechanical ventilation and vasopressor support. (2) Acute sickle cell vaso-occlusive crisis complicated by acute chest syndrome and requiring life-supporting interventions. (3) Sepsis secondary to Streptococcus pneumoniae bacteremia with septic shock requiring vasopressor therapy. (4) Acute kidney injury, KDIGO stage 2, creatinine 2.8 times baseline, resolved without dialysis. (5) Fever, temperature 39.8 degrees Celsius.</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>5/22/96</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M19" s="10" t="inlineStr">
         <is>
           <t>8/10/96</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N19" s="10" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="O19" s="10" t="inlineStr">
         <is>
           <t>Black or African American</t>
         </is>
       </c>
-      <c r="P4" s="4" t="inlineStr"/>
-      <c r="Q4" s="4" t="inlineStr"/>
-      <c r="R4" s="4" t="inlineStr"/>
-      <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr"/>
-      <c r="V4" s="4" t="inlineStr"/>
-      <c r="W4" s="4" t="inlineStr"/>
-      <c r="X4" s="4" t="inlineStr"/>
-      <c r="Y4" s="4" t="inlineStr"/>
-      <c r="Z4" s="4" t="inlineStr"/>
-      <c r="AA4" s="4" t="inlineStr"/>
-      <c r="AB4" s="4" t="inlineStr"/>
-      <c r="AC4" s="4" t="inlineStr"/>
-      <c r="AD4" s="4" t="inlineStr"/>
-      <c r="AE4" s="4" t="inlineStr"/>
-      <c r="AF4" s="4" t="inlineStr"/>
-      <c r="AG4" s="4" t="inlineStr"/>
-      <c r="AH4" s="5" t="inlineStr">
+      <c r="P19" s="12" t="inlineStr"/>
+      <c r="Q19" s="12" t="inlineStr"/>
+      <c r="R19" s="12" t="inlineStr"/>
+      <c r="S19" s="12" t="inlineStr"/>
+      <c r="T19" s="12" t="inlineStr"/>
+      <c r="U19" s="12" t="inlineStr"/>
+      <c r="V19" s="12" t="inlineStr"/>
+      <c r="W19" s="12" t="inlineStr"/>
+      <c r="X19" s="12" t="inlineStr"/>
+      <c r="Y19" s="12" t="inlineStr"/>
+      <c r="Z19" s="12" t="inlineStr"/>
+      <c r="AA19" s="12" t="inlineStr"/>
+      <c r="AB19" s="12" t="inlineStr"/>
+      <c r="AC19" s="12" t="inlineStr"/>
+      <c r="AD19" s="12" t="inlineStr"/>
+      <c r="AE19" s="12" t="inlineStr"/>
+      <c r="AF19" s="12" t="inlineStr"/>
+      <c r="AG19" s="12" t="inlineStr"/>
+      <c r="AH19" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AI4" s="4" t="inlineStr"/>
-      <c r="AJ4" s="4" t="inlineStr"/>
-      <c r="AK4" s="4" t="inlineStr"/>
-      <c r="AL4" s="4" t="inlineStr"/>
-      <c r="AM4" s="4" t="inlineStr"/>
-      <c r="AN4" s="4" t="inlineStr"/>
-      <c r="AO4" s="4" t="inlineStr"/>
-      <c r="AP4" s="4" t="inlineStr"/>
-      <c r="AQ4" s="5" t="inlineStr">
+      <c r="AI19" s="12" t="inlineStr"/>
+      <c r="AJ19" s="12" t="inlineStr"/>
+      <c r="AK19" s="12" t="inlineStr"/>
+      <c r="AL19" s="12" t="inlineStr"/>
+      <c r="AM19" s="12" t="inlineStr"/>
+      <c r="AN19" s="12" t="inlineStr"/>
+      <c r="AO19" s="12" t="inlineStr"/>
+      <c r="AP19" s="12" t="inlineStr"/>
+      <c r="AQ19" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="AR4" s="4" t="inlineStr"/>
-      <c r="AS4" s="4" t="inlineStr"/>
-      <c r="AT4" s="4" t="inlineStr"/>
-      <c r="AU4" s="4" t="inlineStr"/>
-      <c r="AV4" s="4" t="inlineStr"/>
-      <c r="AW4" s="4" t="inlineStr"/>
-      <c r="AX4" s="4" t="inlineStr"/>
-      <c r="AY4" s="5" t="inlineStr">
+      <c r="AR19" s="12" t="inlineStr"/>
+      <c r="AS19" s="12" t="inlineStr"/>
+      <c r="AT19" s="12" t="inlineStr"/>
+      <c r="AU19" s="12" t="inlineStr"/>
+      <c r="AV19" s="12" t="inlineStr"/>
+      <c r="AW19" s="12" t="inlineStr"/>
+      <c r="AX19" s="12" t="inlineStr"/>
+      <c r="AY19" s="13" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AZ4" s="4" t="inlineStr"/>
-      <c r="BA4" s="4" t="inlineStr"/>
-      <c r="BB4" s="4" t="inlineStr"/>
-      <c r="BC4" s="4" t="inlineStr"/>
-      <c r="BD4" s="4" t="inlineStr"/>
-      <c r="BE4" s="4" t="inlineStr"/>
-      <c r="BF4" s="4" t="inlineStr"/>
-      <c r="BG4" s="4" t="inlineStr"/>
-      <c r="BH4" s="4" t="inlineStr"/>
-      <c r="BI4" s="4" t="inlineStr"/>
-      <c r="BJ4" s="4" t="inlineStr"/>
-      <c r="BK4" s="5" t="inlineStr">
+      <c r="AZ19" s="12" t="inlineStr"/>
+      <c r="BA19" s="12" t="inlineStr"/>
+      <c r="BB19" s="12" t="inlineStr"/>
+      <c r="BC19" s="12" t="inlineStr"/>
+      <c r="BD19" s="12" t="inlineStr"/>
+      <c r="BE19" s="12" t="inlineStr"/>
+      <c r="BF19" s="12" t="inlineStr"/>
+      <c r="BG19" s="12" t="inlineStr"/>
+      <c r="BH19" s="12" t="inlineStr"/>
+      <c r="BI19" s="12" t="inlineStr"/>
+      <c r="BJ19" s="12" t="inlineStr"/>
+      <c r="BK19" s="13" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="BL4" s="4" t="inlineStr"/>
-      <c r="BM4" s="4" t="inlineStr"/>
-      <c r="BN4" s="4" t="inlineStr"/>
-      <c r="BO4" s="4" t="inlineStr"/>
-      <c r="BP4" s="4" t="inlineStr"/>
+      <c r="BL19" s="12" t="inlineStr"/>
+      <c r="BM19" s="12" t="inlineStr"/>
+      <c r="BN19" s="12" t="inlineStr"/>
+      <c r="BO19" s="12" t="inlineStr"/>
+      <c r="BP19" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BP4"/>
+  <autoFilter ref="A16:BP19"/>
+  <mergeCells count="14">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1435,7 +1625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1448,72 +1638,192 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Synthetic Notes — Ground-Truth Answer Key</t>
-        </is>
-      </c>
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>📋 ANSWER KEY — HOW TO USE THIS SHEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>WHAT IS THIS?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>This sheet shows the ground-truth grading rationale for every outcome in each synthetic note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Use it to verify that an AI extraction system (e.g., MedGemma) produces the correct grades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO READ EACH ROW</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>• Note ID — Which synthetic note (SYNTH_001, _002, or _003)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>• Outcome &amp; # — The SCOGS outcome name and its number (e.g., Fever = #36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>• Grade — The correct ground-truth grade. Color-coded: green=1, yellow=2, orange=3, red=4, gray=absent</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>• Feature Values — The exact clinical features extracted from the note that feed into the rule engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>• Rule Applied — The specific decision table rule from rules.md that produces this grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>• Key Quote — The verbatim text from the note that supports the feature extraction</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO VERIFY A SYSTEM'S OUTPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>1. Run the system on the note text from the 'Synthetic Notes' sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2. Compare its extracted features against the 'Feature Values' column below</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>3. Compare its assigned grade against the 'Grade' column — mismatches indicate extraction or grading errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>4. If the grade is wrong, check whether the system extracted the right quote (compare 'Key Quote' column)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Note ID</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>Outcome #</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>Feature Values</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Rule Applied</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>Key Quote from Note</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>SYNTH_001
 (Note 1)</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Acute Sickle Cell Pain Episode</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>care_setting = ed_treat_release
 pain_co_complication = false
@@ -1521,125 +1831,125 @@
 death_attributed = false</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>care_setting ≥ clinic AND care_setting &lt; inpatient → Grade 2</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>"Patient monitored in ED for 4 hours with improvement. Not admitted. Discharged home"</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>SYNTH_001
 (Note 1)</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Fever</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D23" s="18" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>temperature = 38.3 °C</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>38.0 ≤ temperature &lt; 38.5 → Grade 1</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>"Temperature 38.3 degrees Celsius (101.0 degrees Fahrenheit)"</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>SYNTH_001
 (Note 1)</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Acute Chest Syndrome</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>#48</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>absent</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>N/A — diagnostic criteria not met</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>No lobar infiltrate on imaging → absent</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>"Chest X-ray: No acute cardiopulmonary disease, no infiltrates"</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="8" t="inlineStr"/>
-      <c r="B7" s="8" t="inlineStr"/>
-      <c r="C7" s="8" t="inlineStr"/>
-      <c r="D7" s="8" t="inlineStr"/>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="16" t="inlineStr"/>
+      <c r="B25" s="16" t="inlineStr"/>
+      <c r="C25" s="16" t="inlineStr"/>
+      <c r="D25" s="16" t="inlineStr"/>
+      <c r="E25" s="16" t="inlineStr"/>
+      <c r="F25" s="16" t="inlineStr"/>
+      <c r="G25" s="16" t="inlineStr"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Acute Sickle Cell Pain Episode</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>care_setting = inpatient
 pain_co_complication = true
@@ -1647,40 +1957,40 @@
 death_attributed = false</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>pain_co_complication = true → Grade 4</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>"Acute sickle cell vaso-occlusive pain crisis complicated by acute chest syndrome"</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="27" ht="60" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Acute Chest Syndrome</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>#48</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D27" s="21" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>fio2_pct = 60%
 resp_support = high_flow
@@ -1688,126 +1998,126 @@
 life_support = false</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>(fio2 ≥ 50 OR resp_support ≥ high_flow OR exchange) AND NOT life_support → Grade 3</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr">
         <is>
           <t>"high-flow nasal cannula at 40 L/min with FiO2 60%"; "Automated red cell exchange performed"</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Fever</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>temperature = 39.2 °C</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>temperature ≥ 38.5 → Grade 2</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>"Temperature 39.2 degrees Celsius (102.6 degrees Fahrenheit)"</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>AKI</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>#19</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>absent</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>creatinine_x_baseline = 1.13
 (below 1.5 threshold)</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>creatinine_x_baseline &lt; 1.5 → absent</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr">
         <is>
           <t>"Serum creatinine 0.9 mg/dL (baseline 0.8 mg/dL, ratio 1.13x baseline)"</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="8" t="inlineStr"/>
-      <c r="B12" s="8" t="inlineStr"/>
-      <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr"/>
-      <c r="E12" s="8" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr"/>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="16" t="inlineStr"/>
+      <c r="B30" s="16" t="inlineStr"/>
+      <c r="C30" s="16" t="inlineStr"/>
+      <c r="D30" s="16" t="inlineStr"/>
+      <c r="E30" s="16" t="inlineStr"/>
+      <c r="F30" s="16" t="inlineStr"/>
+      <c r="G30" s="16" t="inlineStr"/>
+    </row>
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>Acute Sickle Cell Pain Episode</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D31" s="20" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>care_setting = icu
 pain_co_complication = true
@@ -1815,40 +2125,40 @@
 death_attributed = false</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>pain_co_complication OR life_support → Grade 4</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="G31" s="16" t="inlineStr">
         <is>
           <t>"vaso-occlusive crisis complicated by acute chest syndrome and requiring life-supporting interventions"</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="32" ht="60" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
         <is>
           <t>Acute Chest Syndrome</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C32" s="16" t="inlineStr">
         <is>
           <t>#48</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D32" s="20" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E32" s="16" t="inlineStr">
         <is>
           <t>fio2_pct = 100%
 resp_support = invasive_ventilation
@@ -1856,78 +2166,78 @@
 life_support = true</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F32" s="16" t="inlineStr">
         <is>
           <t>(fio2 ≥ 50 OR resp_support ≥ high_flow OR exchange) AND life_support → Grade 4</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="G32" s="16" t="inlineStr">
         <is>
           <t>"FiO2 100%"; "emergently intubated"; "norepinephrine"; "vasopressin"</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>Fever</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E33" s="16" t="inlineStr">
         <is>
           <t>temperature = 39.8 °C</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F33" s="16" t="inlineStr">
         <is>
           <t>temperature ≥ 38.5 → Grade 2</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="G33" s="16" t="inlineStr">
         <is>
           <t>"Temperature 39.8 degrees Celsius (103.6 degrees Fahrenheit)"</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>Acute Kidney Injury</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
         <is>
           <t>#19</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>creatinine_x_baseline = 2.8
 creatinine = 2.8 mg/dL
@@ -1935,102 +2245,147 @@
 esrd_progression = false</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F34" s="16" t="inlineStr">
         <is>
           <t>2.0 ≤ creatinine_x_baseline ≤ 2.9 → Grade 2</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="G34" s="16" t="inlineStr">
         <is>
           <t>"creatinine peaked at 2.8 mg/dL on day 2 (2.8 times baseline of 1.0 mg/dL)"</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>Sepsis</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
         <is>
           <t>#37</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>present*</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Positive blood cultures (S. pneumoniae)
 Vasopressor requirement
 *Grade requires rules.md §37</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>Clinically evident; exact SCOGS grade requires team verification per rules.md §37</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>"blood cultures returned positive for Streptococcus pneumoniae"; "norepinephrine"; "vasopressin"</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
         <is>
           <t>Grade Legend:</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>Grade 1 — Mild</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="B39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="25" t="inlineStr">
         <is>
           <t>Grade 2 — Moderate</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="B40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="26" t="inlineStr">
         <is>
           <t>Grade 3 — Severe</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="B41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="27" t="inlineStr">
         <is>
           <t>Grade 4 — Life-Threatening</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="20" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
+      <c r="B42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t>Grade 5 — Fatal (not used in current notes)</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>Absent — Outcome not present</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="30" t="inlineStr">
+        <is>
+          <t>Present* — Needs team verification</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="25">
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 5 new synthetic notes (SYNTH_004–008), total now 8
New notes expand coverage to 6 distinct outcomes across all 5 SCOGS grades:
- Note 4 (SYNTH_004): Grade 1 Pain — home-managed crisis via telephone
- Note 5 (SYNTH_005): Grade 3 Pain + Grade 2 DVT — new outcome (anticoagulation)
- Note 6 (SYNTH_006): Grade 5 ACS + Pain (FATAL) + Grade 3 AKI (CRRT) — death summary
- Note 7 (SYNTH_007): Grade 1 ACS (room air, antibiotics only) — mildest ACS
- Note 8 (SYNTH_008): Grade 3 Priapism (aspiration/irrigation) — new male-specific outcome

Updated CSV (8 rows), answer key markdown, and Excel workbook with all entries.
</commit_message>
<xml_diff>
--- a/data/synthetic_notes.xlsx
+++ b/data/synthetic_notes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Answer Key" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthetic Notes'!$A$16:$BP$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthetic Notes'!$A$17:$BP$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,6 +68,7 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="12"/>
     </font>
     <font>
@@ -76,13 +77,19 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -151,12 +158,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
-        <bgColor rgb="00BDD7EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C00000"/>
         <bgColor rgb="00C00000"/>
       </patternFill>
@@ -201,12 +202,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,7 +227,6 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -248,17 +248,16 @@
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -624,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP19"/>
+  <dimension ref="A1:BP25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -705,91 +704,97 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>WHAT IS THIS?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>This sheet contains 3 synthetic clinical notes for Sickle Cell Disease patients, formatted in the same</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>This sheet contains 8 synthetic clinical notes for Sickle Cell Disease patients, formatted in the same</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>68-column structure as clincal_notes.csv. Each note has known ground-truth SCOGS grades for testing.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>HOW TO NAVIGATE</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>• Columns A–O (blue) = Patient demographics &amp; clinical note text. Column K has the full note.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>• Columns P–BP (green) = The 53 SCOGS outcome columns. Empty = outcome is absent from the note.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>• Gold-highlighted cells = Outcomes that ARE present, with the SCOGS grade (1–5) as the value.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>• Scroll RIGHT to see all 53 outcome columns. Use Ctrl+Right Arrow to jump to the next graded cell.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>• The header row (row 16) is frozen — it stays visible as you scroll down.</t>
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>• The header row is frozen — it stays visible as you scroll down.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>COLOR KEY</t>
         </is>
@@ -815,400 +820,400 @@
       </c>
       <c r="F15" s="6" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>patient_id</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>visit_datetime</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>facility_type</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>pain_type</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>pain_intensity</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
         <is>
           <t>admitted</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>hemoglobin</t>
         </is>
       </c>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="I17" s="9" t="inlineStr">
         <is>
           <t>oxygen_saturation</t>
         </is>
       </c>
-      <c r="J16" s="9" t="inlineStr">
+      <c r="J17" s="9" t="inlineStr">
         <is>
           <t>weather</t>
         </is>
       </c>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="K17" s="9" t="inlineStr">
         <is>
           <t>clinical_note</t>
         </is>
       </c>
-      <c r="L16" s="9" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
         <is>
           <t>dob</t>
         </is>
       </c>
-      <c r="M16" s="9" t="inlineStr">
+      <c r="M17" s="9" t="inlineStr">
         <is>
           <t>diagnosis_date</t>
         </is>
       </c>
-      <c r="N16" s="9" t="inlineStr">
+      <c r="N17" s="9" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="O16" s="9" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>race</t>
         </is>
       </c>
-      <c r="P16" s="9" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr">
         <is>
           <t>arrhythmia</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>deep_vein_thrombosis_dvt</t>
         </is>
       </c>
-      <c r="R16" s="9" t="inlineStr">
+      <c r="R17" s="9" t="inlineStr">
         <is>
           <t>diastolic_dysfunction</t>
         </is>
       </c>
-      <c r="S16" s="9" t="inlineStr">
+      <c r="S17" s="9" t="inlineStr">
         <is>
           <t>heart_failure_exacerbation</t>
         </is>
       </c>
-      <c r="T16" s="9" t="inlineStr">
+      <c r="T17" s="9" t="inlineStr">
         <is>
           <t>myocardial_infarction</t>
         </is>
       </c>
-      <c r="U16" s="9" t="inlineStr">
+      <c r="U17" s="9" t="inlineStr">
         <is>
           <t>systemic_arterial_hypertension</t>
         </is>
       </c>
-      <c r="V16" s="9" t="inlineStr">
+      <c r="V17" s="9" t="inlineStr">
         <is>
           <t>systolic_dysfunction</t>
         </is>
       </c>
-      <c r="W16" s="9" t="inlineStr">
+      <c r="W17" s="9" t="inlineStr">
         <is>
           <t>tricuspid_regurgitant_jet_velocity_trv_elevation_on_echocardiogram</t>
         </is>
       </c>
-      <c r="X16" s="9" t="inlineStr">
+      <c r="X17" s="9" t="inlineStr">
         <is>
           <t>cerebral_vasculopathy</t>
         </is>
       </c>
-      <c r="Y16" s="9" t="inlineStr">
+      <c r="Y17" s="9" t="inlineStr">
         <is>
           <t>chronic_pain</t>
         </is>
       </c>
-      <c r="Z16" s="9" t="inlineStr">
+      <c r="Z17" s="9" t="inlineStr">
         <is>
           <t>cognitive_dysfunction</t>
         </is>
       </c>
-      <c r="AA16" s="9" t="inlineStr">
+      <c r="AA17" s="9" t="inlineStr">
         <is>
           <t>elevated_transcranial_doppler_tcd_ultrasonography_velocity</t>
         </is>
       </c>
-      <c r="AB16" s="9" t="inlineStr">
+      <c r="AB17" s="9" t="inlineStr">
         <is>
           <t>posterior_reversible_encephalopathy_syndrome_pres</t>
         </is>
       </c>
-      <c r="AC16" s="9" t="inlineStr">
+      <c r="AC17" s="9" t="inlineStr">
         <is>
           <t>silent_cerebral_infarct</t>
         </is>
       </c>
-      <c r="AD16" s="9" t="inlineStr">
+      <c r="AD17" s="9" t="inlineStr">
         <is>
           <t>stroke_hemorrhagic_or_ischemic</t>
         </is>
       </c>
-      <c r="AE16" s="9" t="inlineStr">
+      <c r="AE17" s="9" t="inlineStr">
         <is>
           <t>hearing_loss_in_at_least_one_ear</t>
         </is>
       </c>
-      <c r="AF16" s="9" t="inlineStr">
+      <c r="AF17" s="9" t="inlineStr">
         <is>
           <t>sickle_cell_retinopathy_scr</t>
         </is>
       </c>
-      <c r="AG16" s="9" t="inlineStr">
+      <c r="AG17" s="9" t="inlineStr">
         <is>
           <t>cholecystitis_cholelithiasis_gallstones</t>
         </is>
       </c>
-      <c r="AH16" s="9" t="inlineStr">
+      <c r="AH17" s="9" t="inlineStr">
         <is>
           <t>acute_kidney_injury_aki</t>
         </is>
       </c>
-      <c r="AI16" s="9" t="inlineStr">
+      <c r="AI17" s="9" t="inlineStr">
         <is>
           <t>acute_papillary_necrosis</t>
         </is>
       </c>
-      <c r="AJ16" s="9" t="inlineStr">
+      <c r="AJ17" s="9" t="inlineStr">
         <is>
           <t>chronic_kidney_disease_ckd</t>
         </is>
       </c>
-      <c r="AK16" s="9" t="inlineStr">
+      <c r="AK17" s="9" t="inlineStr">
         <is>
           <t>female_ovarian_dysfunction</t>
         </is>
       </c>
-      <c r="AL16" s="9" t="inlineStr">
+      <c r="AL17" s="9" t="inlineStr">
         <is>
           <t>male_impairments</t>
         </is>
       </c>
-      <c r="AM16" s="9" t="inlineStr">
+      <c r="AM17" s="9" t="inlineStr">
         <is>
           <t>priapism</t>
         </is>
       </c>
-      <c r="AN16" s="9" t="inlineStr">
+      <c r="AN17" s="9" t="inlineStr">
         <is>
           <t>delayed_puberty</t>
         </is>
       </c>
-      <c r="AO16" s="9" t="inlineStr">
+      <c r="AO17" s="9" t="inlineStr">
         <is>
           <t>malnutrition_leading_to_stunting_decreased_height_velocity</t>
         </is>
       </c>
-      <c r="AP16" s="9" t="inlineStr">
+      <c r="AP17" s="9" t="inlineStr">
         <is>
           <t>underweight</t>
         </is>
       </c>
-      <c r="AQ16" s="9" t="inlineStr">
+      <c r="AQ17" s="9" t="inlineStr">
         <is>
           <t>acute_sickle_cell_pain_episode</t>
         </is>
       </c>
-      <c r="AR16" s="9" t="inlineStr">
+      <c r="AR17" s="9" t="inlineStr">
         <is>
           <t>acute_splenic_sequestration</t>
         </is>
       </c>
-      <c r="AS16" s="9" t="inlineStr">
+      <c r="AS17" s="9" t="inlineStr">
         <is>
           <t>alloimmunization_delayed_hemolytic_transfusion_reaction_dhtr</t>
         </is>
       </c>
-      <c r="AT16" s="9" t="inlineStr">
+      <c r="AT17" s="9" t="inlineStr">
         <is>
           <t>chronic_hypersplenism</t>
         </is>
       </c>
-      <c r="AU16" s="9" t="inlineStr">
+      <c r="AU17" s="9" t="inlineStr">
         <is>
           <t>hepatopathy</t>
         </is>
       </c>
-      <c r="AV16" s="9" t="inlineStr">
+      <c r="AV17" s="9" t="inlineStr">
         <is>
           <t>splenic_infarction</t>
         </is>
       </c>
-      <c r="AW16" s="9" t="inlineStr">
+      <c r="AW17" s="9" t="inlineStr">
         <is>
           <t>transfusional_iron_overload_hemochromatosis_or_hemosiderosis</t>
         </is>
       </c>
-      <c r="AX16" s="9" t="inlineStr">
+      <c r="AX17" s="9" t="inlineStr">
         <is>
           <t>transient_aplastic_crisis_secondary_to_parvovirus_b19_infection</t>
         </is>
       </c>
-      <c r="AY16" s="9" t="inlineStr">
+      <c r="AY17" s="9" t="inlineStr">
         <is>
           <t>fever</t>
         </is>
       </c>
-      <c r="AZ16" s="9" t="inlineStr">
+      <c r="AZ17" s="9" t="inlineStr">
         <is>
           <t>sepsis</t>
         </is>
       </c>
-      <c r="BA16" s="9" t="inlineStr">
+      <c r="BA17" s="9" t="inlineStr">
         <is>
           <t>malignant_neoplasms</t>
         </is>
       </c>
-      <c r="BB16" s="9" t="inlineStr">
+      <c r="BB17" s="9" t="inlineStr">
         <is>
           <t>avascular_necrosis_of_joints_avn</t>
         </is>
       </c>
-      <c r="BC16" s="9" t="inlineStr">
+      <c r="BC17" s="9" t="inlineStr">
         <is>
           <t>leg_ulcer</t>
         </is>
       </c>
-      <c r="BD16" s="9" t="inlineStr">
+      <c r="BD17" s="9" t="inlineStr">
         <is>
           <t>osteomyelitis</t>
         </is>
       </c>
-      <c r="BE16" s="9" t="inlineStr">
+      <c r="BE17" s="9" t="inlineStr">
         <is>
           <t>osteoporosis</t>
         </is>
       </c>
-      <c r="BF16" s="9" t="inlineStr">
+      <c r="BF17" s="9" t="inlineStr">
         <is>
           <t>acute_multiorgan_failure</t>
         </is>
       </c>
-      <c r="BG16" s="9" t="inlineStr">
+      <c r="BG17" s="9" t="inlineStr">
         <is>
           <t>fetal_growth_restriction</t>
         </is>
       </c>
-      <c r="BH16" s="9" t="inlineStr">
+      <c r="BH17" s="9" t="inlineStr">
         <is>
           <t>pregnancy_loss</t>
         </is>
       </c>
-      <c r="BI16" s="9" t="inlineStr">
+      <c r="BI17" s="9" t="inlineStr">
         <is>
           <t>premature_delivery</t>
         </is>
       </c>
-      <c r="BJ16" s="9" t="inlineStr">
+      <c r="BJ17" s="9" t="inlineStr">
         <is>
           <t>depression</t>
         </is>
       </c>
-      <c r="BK16" s="9" t="inlineStr">
+      <c r="BK17" s="9" t="inlineStr">
         <is>
           <t>acute_chest_syndrome_acs</t>
         </is>
       </c>
-      <c r="BL16" s="9" t="inlineStr">
+      <c r="BL17" s="9" t="inlineStr">
         <is>
           <t>asthma_exacerbation</t>
         </is>
       </c>
-      <c r="BM16" s="9" t="inlineStr">
+      <c r="BM17" s="9" t="inlineStr">
         <is>
           <t>chronic_restrictive_lung_physiology</t>
         </is>
       </c>
-      <c r="BN16" s="9" t="inlineStr">
+      <c r="BN17" s="9" t="inlineStr">
         <is>
           <t>pulmonary_embolism_pe</t>
         </is>
       </c>
-      <c r="BO16" s="9" t="inlineStr">
+      <c r="BO17" s="9" t="inlineStr">
         <is>
           <t>pulmonary_hypertension</t>
         </is>
       </c>
-      <c r="BP16" s="9" t="inlineStr">
+      <c r="BP17" s="9" t="inlineStr">
         <is>
           <t>sleep_apnea_obstructive_or_central</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="200" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18" ht="200" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>SYNTH_001</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>3/15/25</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>ER</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Leg Pain</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Memphis</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>7.8</t>
         </is>
       </c>
-      <c r="I17" s="10" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>98</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>Warm</t>
         </is>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>SUBJECTIVE: 22-year-old female with known sickle cell disease (HbSS), diagnosed at age 2, presents to the emergency department with bilateral lower extremity pain that began approximately 6 hours ago. She describes the pain as deep, aching, and throbbing, rated 7 out of 10 in intensity. She reports taking ibuprofen 600 mg and acetaminophen 1000 mg at home without adequate relief. She also notes feeling warm and mildly fatigued. She denies cough, shortness of breath, chest pain, abdominal pain, headache, vision changes, or urinary symptoms. No recent travel or sick contacts. No history of DVT or pulmonary embolism.
 OBJECTIVE: Temperature 38.3 degrees Celsius (101.0 degrees Fahrenheit), heart rate 98 bpm, blood pressure 112/68 mmHg, respiratory rate 18 breaths/min, SpO2 98% on room air. General: Alert, oriented, appears uncomfortable but not in acute distress. HEENT: Scleral icterus noted bilaterally. Lungs: Clear to auscultation bilaterally, no wheezes, crackles, or rhonchi. Cardiovascular: Regular rate and rhythm, no murmurs, rubs, or gallops. Abdomen: Soft, non-tender, non-distended, no hepatosplenomegaly. Extremities: Bilateral tibial tenderness to palpation without swelling or erythema, no edema, no calf tenderness, no leg ulcers. Neurological: Alert and oriented x4, cranial nerves II-XII intact, no focal motor or sensory deficits, gait not assessed due to pain.
@@ -1216,162 +1221,19 @@
 ASSESSMENT AND PLAN: (1) Acute sickle cell vaso-occlusive pain episode. Administered IV normal saline bolus 1 liter, IV morphine 4 mg with adequate pain relief achieved (pain reduced to 3/10). Patient monitored in ED for 4 hours with improvement. Not admitted. Discharged home with oral oxycodone 5 mg every 4-6 hours as needed for pain, ibuprofen 600 mg every 8 hours, and instructions to return if fever exceeds 38.5 degrees Celsius, or if she develops chest pain, shortness of breath, or worsening symptoms. Follow-up with hematology clinic in 48 hours. (2) Low-grade fever, temperature 38.3 degrees Celsius. Most likely related to vaso-occlusive crisis. Blood cultures pending. No signs of acute chest syndrome, sepsis, or other infectious source identified.</t>
         </is>
       </c>
-      <c r="L17" s="10" t="inlineStr">
+      <c r="L18" s="10" t="inlineStr">
         <is>
           <t>4/10/03</t>
         </is>
       </c>
-      <c r="M17" s="10" t="inlineStr">
+      <c r="M18" s="10" t="inlineStr">
         <is>
           <t>6/20/05</t>
         </is>
       </c>
-      <c r="N17" s="10" t="inlineStr">
+      <c r="N18" s="10" t="inlineStr">
         <is>
           <t>Female</t>
-        </is>
-      </c>
-      <c r="O17" s="10" t="inlineStr">
-        <is>
-          <t>Black or African American</t>
-        </is>
-      </c>
-      <c r="P17" s="12" t="inlineStr"/>
-      <c r="Q17" s="12" t="inlineStr"/>
-      <c r="R17" s="12" t="inlineStr"/>
-      <c r="S17" s="12" t="inlineStr"/>
-      <c r="T17" s="12" t="inlineStr"/>
-      <c r="U17" s="12" t="inlineStr"/>
-      <c r="V17" s="12" t="inlineStr"/>
-      <c r="W17" s="12" t="inlineStr"/>
-      <c r="X17" s="12" t="inlineStr"/>
-      <c r="Y17" s="12" t="inlineStr"/>
-      <c r="Z17" s="12" t="inlineStr"/>
-      <c r="AA17" s="12" t="inlineStr"/>
-      <c r="AB17" s="12" t="inlineStr"/>
-      <c r="AC17" s="12" t="inlineStr"/>
-      <c r="AD17" s="12" t="inlineStr"/>
-      <c r="AE17" s="12" t="inlineStr"/>
-      <c r="AF17" s="12" t="inlineStr"/>
-      <c r="AG17" s="12" t="inlineStr"/>
-      <c r="AH17" s="12" t="inlineStr"/>
-      <c r="AI17" s="12" t="inlineStr"/>
-      <c r="AJ17" s="12" t="inlineStr"/>
-      <c r="AK17" s="12" t="inlineStr"/>
-      <c r="AL17" s="12" t="inlineStr"/>
-      <c r="AM17" s="12" t="inlineStr"/>
-      <c r="AN17" s="12" t="inlineStr"/>
-      <c r="AO17" s="12" t="inlineStr"/>
-      <c r="AP17" s="12" t="inlineStr"/>
-      <c r="AQ17" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="AR17" s="12" t="inlineStr"/>
-      <c r="AS17" s="12" t="inlineStr"/>
-      <c r="AT17" s="12" t="inlineStr"/>
-      <c r="AU17" s="12" t="inlineStr"/>
-      <c r="AV17" s="12" t="inlineStr"/>
-      <c r="AW17" s="12" t="inlineStr"/>
-      <c r="AX17" s="12" t="inlineStr"/>
-      <c r="AY17" s="13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AZ17" s="12" t="inlineStr"/>
-      <c r="BA17" s="12" t="inlineStr"/>
-      <c r="BB17" s="12" t="inlineStr"/>
-      <c r="BC17" s="12" t="inlineStr"/>
-      <c r="BD17" s="12" t="inlineStr"/>
-      <c r="BE17" s="12" t="inlineStr"/>
-      <c r="BF17" s="12" t="inlineStr"/>
-      <c r="BG17" s="12" t="inlineStr"/>
-      <c r="BH17" s="12" t="inlineStr"/>
-      <c r="BI17" s="12" t="inlineStr"/>
-      <c r="BJ17" s="12" t="inlineStr"/>
-      <c r="BK17" s="12" t="inlineStr"/>
-      <c r="BL17" s="12" t="inlineStr"/>
-      <c r="BM17" s="12" t="inlineStr"/>
-      <c r="BN17" s="12" t="inlineStr"/>
-      <c r="BO17" s="12" t="inlineStr"/>
-      <c r="BP17" s="12" t="inlineStr"/>
-    </row>
-    <row r="18" ht="200" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>SYNTH_002</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>7/22/25</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>ER</t>
-        </is>
-      </c>
-      <c r="D18" s="10" t="inlineStr">
-        <is>
-          <t>Chest Pain</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>Memphis</t>
-        </is>
-      </c>
-      <c r="G18" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>6.2</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>88</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>Hot</t>
-        </is>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>SUBJECTIVE: 17-year-old male with sickle cell disease (HbSS), on chronic transfusion program, presents with acute onset of severe generalized body pain rated 9 out of 10, productive cough with yellowish sputum, and progressive shortness of breath over the past 18 hours. He reports fever at home measured at 39.2 degrees Celsius (102.6 degrees Fahrenheit). He has had three prior hospitalizations for acute chest syndrome in the past two years. He denies headache, visual changes, abdominal pain, dysuria, or hematuria. No history of leg swelling, DVT, or pulmonary embolism. No depressive symptoms reported.
-OBJECTIVE: Temperature 39.2 degrees Celsius (102.6 degrees Fahrenheit), heart rate 118 bpm, blood pressure 102/58 mmHg, respiratory rate 28 breaths/min, SpO2 88% on room air. General: Acutely ill-appearing, diaphoretic, using accessory muscles of respiration. HEENT: Scleral icterus, dry mucous membranes. Lungs: Decreased breath sounds at right lower lobe with dullness to percussion and bronchial breath sounds; scattered crackles bilaterally. Cardiovascular: Tachycardic, regular rhythm, grade II/VI systolic flow murmur at left sternal border. Abdomen: Mild splenomegaly palpated 2 cm below left costal margin, no acute tenderness. Extremities: Diffuse tenderness in bilateral upper and lower extremities, no edema, no calf tenderness, no leg ulcers. Neurological: Alert and oriented x3, no focal neurological deficits, moving all extremities symmetrically, cranial nerves intact.
-LABS: Hemoglobin 6.2 g/dL (baseline 9.0 g/dL), WBC 18.7 x 10^3/uL with 8% bands, platelets 198 x 10^3/uL, reticulocyte count 12.1%. HbS level 78%. Serum creatinine 0.9 mg/dL (baseline 0.8 mg/dL, ratio 1.13x baseline). LDH 687 U/L, total bilirubin 5.8 mg/dL, AST 62 U/L, ALT 38 U/L. ABG: pH 7.38, PaCO2 32 mmHg, PaO2 58 mmHg on room air. Blood cultures obtained; pending at time of admission. Chest X-ray: New right lower lobe consolidation with air bronchograms consistent with a new lobar infiltrate. No pleural effusion. CT pulmonary angiography: No evidence of pulmonary embolism; confirmed right lower lobe consolidation.
-HOSPITAL COURSE: Patient admitted to the medical floor. Initiated on ceftriaxone 2 g IV daily and azithromycin 500 mg IV for empiric coverage of acute chest syndrome. IV morphine PCA established for pain management. Initially placed on supplemental oxygen via nasal cannula at 4 L/min (FiO2 approximately 36%), achieving SpO2 of 92%. On hospital day 2, respiratory status worsened with increasing tachypnea (RR 34) and SpO2 dropping to 84% on nasal cannula. Transitioned to high-flow nasal cannula at 40 L/min with FiO2 60%, achieving SpO2 of 93%. Patient did not require intubation, vasopressors, or other life-support interventions. Hematology consulted and recommended urgent exchange transfusion due to progressive acute chest syndrome. Automated red cell exchange performed, reducing HbS from 78% to 28%, with post-procedure hemoglobin of 10.1 g/dL. Patient demonstrated significant clinical improvement over the following 48 hours. Weaned to low-flow nasal cannula by day 4 and to room air by day 5. Pain gradually improved and PCA discontinued on day 4, transitioned to oral analgesics.
-DISCHARGE SUMMARY: Temperature normalized by hospital day 3. Blood cultures returned negative. Repeat chest X-ray showed improving right lower lobe infiltrate. Serum creatinine remained stable at 0.9 mg/dL throughout admission. No evidence of DVT on bilateral lower extremity Doppler ultrasound. No neurological complications observed. No arrhythmias noted on telemetry monitoring. Discharged on hospital day 7 in stable condition with follow-up in sickle cell clinic in one week.
-DISCHARGE DIAGNOSES: (1) Acute chest syndrome, severe, requiring high-flow oxygen therapy and exchange transfusion. (2) Acute sickle cell vaso-occlusive pain crisis complicated by acute chest syndrome. (3) Fever secondary to acute chest syndrome.</t>
-        </is>
-      </c>
-      <c r="L18" s="10" t="inlineStr">
-        <is>
-          <t>11/3/07</t>
-        </is>
-      </c>
-      <c r="M18" s="10" t="inlineStr">
-        <is>
-          <t>2/15/08</t>
-        </is>
-      </c>
-      <c r="N18" s="10" t="inlineStr">
-        <is>
-          <t>Male</t>
         </is>
       </c>
       <c r="O18" s="10" t="inlineStr">
@@ -1408,7 +1270,7 @@
       <c r="AP18" s="12" t="inlineStr"/>
       <c r="AQ18" s="13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AR18" s="12" t="inlineStr"/>
@@ -1420,7 +1282,7 @@
       <c r="AX18" s="12" t="inlineStr"/>
       <c r="AY18" s="13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="AZ18" s="12" t="inlineStr"/>
@@ -1434,11 +1296,7 @@
       <c r="BH18" s="12" t="inlineStr"/>
       <c r="BI18" s="12" t="inlineStr"/>
       <c r="BJ18" s="12" t="inlineStr"/>
-      <c r="BK18" s="13" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="BK18" s="12" t="inlineStr"/>
       <c r="BL18" s="12" t="inlineStr"/>
       <c r="BM18" s="12" t="inlineStr"/>
       <c r="BN18" s="12" t="inlineStr"/>
@@ -1448,12 +1306,12 @@
     <row r="19" ht="200" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>SYNTH_003</t>
+          <t>SYNTH_002</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>1/8/26</t>
+          <t>7/22/25</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -1468,7 +1326,7 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
@@ -1483,38 +1341,37 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>88</t>
         </is>
       </c>
       <c r="J19" s="10" t="inlineStr">
         <is>
-          <t>Cold</t>
+          <t>Hot</t>
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>SUBJECTIVE: 29-year-old male with sickle cell disease (HbSC), known history of avascular necrosis of the right hip (managed conservatively), presents via EMS to the emergency department with acute severe chest pain, progressive dyspnea, and high-grade fever for the past 8 hours. His wife reports he had been experiencing a vaso-occlusive pain crisis at home for two days managed with oral hydromorphone, but acutely worsened with onset of chest pain and difficulty breathing. She notes he became confused and less responsive during transport. No prior history of stroke, DVT, or PE. No psychiatric history or depressive symptoms.
-OBJECTIVE: Temperature 39.8 degrees Celsius (103.6 degrees Fahrenheit), heart rate 132 bpm, blood pressure 78/42 mmHg, respiratory rate 36 breaths/min, SpO2 79% on 15 L non-rebreather mask. General: Critically ill-appearing, obtunded, diaphoretic, severe respiratory distress with use of accessory muscles, intercostal and suprasternal retractions. HEENT: Scleral icterus, dry mucous membranes. Lungs: Diffuse bilateral crackles with diminished breath sounds in bilateral lower lobes. Cardiovascular: Tachycardic, distant heart sounds, no appreciable murmur. Abdomen: Distended, diffusely tender, hepatomegaly palpated 4 cm below right costal margin. Extremities: Cool, mottled, capillary refill greater than 4 seconds bilaterally, no peripheral edema, no leg ulcers. Neurological: GCS 10 (E2 V3 M5), pupils 3 mm bilaterally and reactive, withdraws to pain in all extremities. No lateralizing signs.
-LABS: Hemoglobin 5.1 g/dL (baseline 11.5 g/dL), WBC 24.3 x 10^3/uL with 15% bands, platelets 89 x 10^3/uL, reticulocyte count 14.2%. HbS level 52%. Serum creatinine 2.4 mg/dL (baseline 1.0 mg/dL, 2.4x baseline). BUN 38 mg/dL. LDH 1247 U/L, total bilirubin 9.6 mg/dL, direct bilirubin 4.2 mg/dL, AST 189 U/L, ALT 94 U/L. Lactate 6.8 mmol/L. Procalcitonin 8.4 ng/mL. ABG: pH 7.22, PaCO2 28 mmHg, PaO2 48 mmHg on 15 L NRB. Coagulation: INR 1.8, aPTT 42 seconds. Blood cultures: Two sets drawn from peripheral sites. Chest X-ray: Bilateral diffuse alveolar infiltrates with consolidation in all lobes, small bilateral pleural effusions. CT pulmonary angiography: No evidence of pulmonary embolism; confirmed bilateral multilobar consolidations consistent with acute chest syndrome. Lower extremity Doppler ultrasound: No evidence of deep vein thrombosis. Urine output: 15 mL in the first 2 hours (oliguria).
-ICU COURSE: Patient emergently intubated in the ED for acute hypoxemic respiratory failure with deteriorating mental status (GCS 10). Post-intubation ventilator settings: assist-control mode, FiO2 100%, PEEP 10 cmH2O, tidal volume 400 mL (6 mL/kg IBW). Aggressive fluid resuscitation initiated with 30 mL/kg crystalloid bolus. Despite 2 liters of IV normal saline, blood pressure remained 72/38 mmHg with MAP 49. Central venous catheter placed in the right internal jugular vein and norepinephrine infusion started at 0.15 mcg/kg/min, titrated to 0.3 mcg/kg/min to achieve MAP greater than 65 mmHg. Vasopressin 0.04 units/min added as a second vasopressor. Broad-spectrum antibiotics initiated: vancomycin 1.5 g IV, meropenem 1 g IV every 8 hours, and azithromycin 500 mg IV daily. Urgent automated red cell exchange transfusion performed, reducing HbS from 52% to 18%, with post-exchange hemoglobin of 9.8 g/dL.
-On ICU day 2, blood cultures returned positive for Streptococcus pneumoniae in both sets; antibiotics narrowed to ceftriaxone based on susceptibilities. Repeat ABG showed improvement: pH 7.31, PaCO2 34 mmHg, PaO2 72 mmHg on FiO2 80%. Serum creatinine peaked at 2.8 mg/dL on day 2 (2.8 times baseline of 1.0 mg/dL). Urine output improved to 0.5 mL/kg/hr after hemodynamic stabilization; renal replacement therapy was not required. By ICU day 4, vasopressors successfully weaned off and FiO2 reduced to 50%. Extubated on ICU day 6 to high-flow nasal cannula, then weaned to room air by day 8. Transferred to medical floor on day 7. Mental status returned to baseline. No seizures or focal neurological deficits observed throughout admission. No arrhythmias on continuous telemetry.
-DISCHARGE SUMMARY: Creatinine normalized to 1.1 mg/dL by discharge. Repeat chest X-ray showed near-complete resolution of bilateral infiltrates. No evidence of pulmonary embolism, stroke, or other neurological complications. Hearing intact bilaterally. PHQ-9 score 3 (minimal depression). Patient discharged on hospital day 14 in stable condition with close hematology follow-up.
-DISCHARGE DIAGNOSES: (1) Acute chest syndrome, life-threatening, requiring invasive mechanical ventilation and vasopressor support. (2) Acute sickle cell vaso-occlusive crisis complicated by acute chest syndrome and requiring life-supporting interventions. (3) Sepsis secondary to Streptococcus pneumoniae bacteremia with septic shock requiring vasopressor therapy. (4) Acute kidney injury, KDIGO stage 2, creatinine 2.8 times baseline, resolved without dialysis. (5) Fever, temperature 39.8 degrees Celsius.</t>
+          <t>SUBJECTIVE: 17-year-old male with sickle cell disease (HbSS), on chronic transfusion program, presents with acute onset of severe generalized body pain rated 9 out of 10, productive cough with yellowish sputum, and progressive shortness of breath over the past 18 hours. He reports fever at home measured at 39.2 degrees Celsius (102.6 degrees Fahrenheit). He has had three prior hospitalizations for acute chest syndrome in the past two years. He denies headache, visual changes, abdominal pain, dysuria, or hematuria. No history of leg swelling, DVT, or pulmonary embolism. No depressive symptoms reported.
+OBJECTIVE: Temperature 39.2 degrees Celsius (102.6 degrees Fahrenheit), heart rate 118 bpm, blood pressure 102/58 mmHg, respiratory rate 28 breaths/min, SpO2 88% on room air. General: Acutely ill-appearing, diaphoretic, using accessory muscles of respiration. HEENT: Scleral icterus, dry mucous membranes. Lungs: Decreased breath sounds at right lower lobe with dullness to percussion and bronchial breath sounds; scattered crackles bilaterally. Cardiovascular: Tachycardic, regular rhythm, grade II/VI systolic flow murmur at left sternal border. Abdomen: Mild splenomegaly palpated 2 cm below left costal margin, no acute tenderness. Extremities: Diffuse tenderness in bilateral upper and lower extremities, no edema, no calf tenderness, no leg ulcers. Neurological: Alert and oriented x3, no focal neurological deficits, moving all extremities symmetrically, cranial nerves intact.
+LABS: Hemoglobin 6.2 g/dL (baseline 9.0 g/dL), WBC 18.7 x 10^3/uL with 8% bands, platelets 198 x 10^3/uL, reticulocyte count 12.1%. HbS level 78%. Serum creatinine 0.9 mg/dL (baseline 0.8 mg/dL, ratio 1.13x baseline). LDH 687 U/L, total bilirubin 5.8 mg/dL, AST 62 U/L, ALT 38 U/L. ABG: pH 7.38, PaCO2 32 mmHg, PaO2 58 mmHg on room air. Blood cultures obtained; pending at time of admission. Chest X-ray: New right lower lobe consolidation with air bronchograms consistent with a new lobar infiltrate. No pleural effusion. CT pulmonary angiography: No evidence of pulmonary embolism; confirmed right lower lobe consolidation.
+HOSPITAL COURSE: Patient admitted to the medical floor. Initiated on ceftriaxone 2 g IV daily and azithromycin 500 mg IV for empiric coverage of acute chest syndrome. IV morphine PCA established for pain management. Initially placed on supplemental oxygen via nasal cannula at 4 L/min (FiO2 approximately 36%), achieving SpO2 of 92%. On hospital day 2, respiratory status worsened with increasing tachypnea (RR 34) and SpO2 dropping to 84% on nasal cannula. Transitioned to high-flow nasal cannula at 40 L/min with FiO2 60%, achieving SpO2 of 93%. Patient did not require intubation, vasopressors, or other life-support interventions. Hematology consulted and recommended urgent exchange transfusion due to progressive acute chest syndrome. Automated red cell exchange performed, reducing HbS from 78% to 28%, with post-procedure hemoglobin of 10.1 g/dL. Patient demonstrated significant clinical improvement over the following 48 hours. Weaned to low-flow nasal cannula by day 4 and to room air by day 5. Pain gradually improved and PCA discontinued on day 4, transitioned to oral analgesics.
+DISCHARGE SUMMARY: Temperature normalized by hospital day 3. Blood cultures returned negative. Repeat chest X-ray showed improving right lower lobe infiltrate. Serum creatinine remained stable at 0.9 mg/dL throughout admission. No evidence of DVT on bilateral lower extremity Doppler ultrasound. No neurological complications observed. No arrhythmias noted on telemetry monitoring. Discharged on hospital day 7 in stable condition with follow-up in sickle cell clinic in one week.
+DISCHARGE DIAGNOSES: (1) Acute chest syndrome, severe, requiring high-flow oxygen therapy and exchange transfusion. (2) Acute sickle cell vaso-occlusive pain crisis complicated by acute chest syndrome. (3) Fever secondary to acute chest syndrome.</t>
         </is>
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
-          <t>5/22/96</t>
+          <t>11/3/07</t>
         </is>
       </c>
       <c r="M19" s="10" t="inlineStr">
         <is>
-          <t>8/10/96</t>
+          <t>2/15/08</t>
         </is>
       </c>
       <c r="N19" s="10" t="inlineStr">
@@ -1545,11 +1402,7 @@
       <c r="AE19" s="12" t="inlineStr"/>
       <c r="AF19" s="12" t="inlineStr"/>
       <c r="AG19" s="12" t="inlineStr"/>
-      <c r="AH19" s="13" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="AH19" s="12" t="inlineStr"/>
       <c r="AI19" s="12" t="inlineStr"/>
       <c r="AJ19" s="12" t="inlineStr"/>
       <c r="AK19" s="12" t="inlineStr"/>
@@ -1588,7 +1441,7 @@
       <c r="BJ19" s="12" t="inlineStr"/>
       <c r="BK19" s="13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="BL19" s="12" t="inlineStr"/>
@@ -1597,8 +1450,896 @@
       <c r="BO19" s="12" t="inlineStr"/>
       <c r="BP19" s="12" t="inlineStr"/>
     </row>
+    <row r="20" ht="200" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_003</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>1/8/26</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>Chest Pain</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 29-year-old male with sickle cell disease (HbSC), known history of avascular necrosis of the right hip (managed conservatively), presents via EMS to the emergency department with acute severe chest pain, progressive dyspnea, and high-grade fever for the past 8 hours. His wife reports he had been experiencing a vaso-occlusive pain crisis at home for two days managed with oral hydromorphone, but acutely worsened with onset of chest pain and difficulty breathing. She notes he became confused and less responsive during transport. No prior history of stroke, DVT, or PE. No psychiatric history or depressive symptoms.
+OBJECTIVE: Temperature 39.8 degrees Celsius (103.6 degrees Fahrenheit), heart rate 132 bpm, blood pressure 78/42 mmHg, respiratory rate 36 breaths/min, SpO2 79% on 15 L non-rebreather mask. General: Critically ill-appearing, obtunded, diaphoretic, severe respiratory distress with use of accessory muscles, intercostal and suprasternal retractions. HEENT: Scleral icterus, dry mucous membranes. Lungs: Diffuse bilateral crackles with diminished breath sounds in bilateral lower lobes. Cardiovascular: Tachycardic, distant heart sounds, no appreciable murmur. Abdomen: Distended, diffusely tender, hepatomegaly palpated 4 cm below right costal margin. Extremities: Cool, mottled, capillary refill greater than 4 seconds bilaterally, no peripheral edema, no leg ulcers. Neurological: GCS 10 (E2 V3 M5), pupils 3 mm bilaterally and reactive, withdraws to pain in all extremities. No lateralizing signs.
+LABS: Hemoglobin 5.1 g/dL (baseline 11.5 g/dL), WBC 24.3 x 10^3/uL with 15% bands, platelets 89 x 10^3/uL, reticulocyte count 14.2%. HbS level 52%. Serum creatinine 2.4 mg/dL (baseline 1.0 mg/dL, 2.4x baseline). BUN 38 mg/dL. LDH 1247 U/L, total bilirubin 9.6 mg/dL, direct bilirubin 4.2 mg/dL, AST 189 U/L, ALT 94 U/L. Lactate 6.8 mmol/L. Procalcitonin 8.4 ng/mL. ABG: pH 7.22, PaCO2 28 mmHg, PaO2 48 mmHg on 15 L NRB. Coagulation: INR 1.8, aPTT 42 seconds. Blood cultures: Two sets drawn from peripheral sites. Chest X-ray: Bilateral diffuse alveolar infiltrates with consolidation in all lobes, small bilateral pleural effusions. CT pulmonary angiography: No evidence of pulmonary embolism; confirmed bilateral multilobar consolidations consistent with acute chest syndrome. Lower extremity Doppler ultrasound: No evidence of deep vein thrombosis. Urine output: 15 mL in the first 2 hours (oliguria).
+ICU COURSE: Patient emergently intubated in the ED for acute hypoxemic respiratory failure with deteriorating mental status (GCS 10). Post-intubation ventilator settings: assist-control mode, FiO2 100%, PEEP 10 cmH2O, tidal volume 400 mL (6 mL/kg IBW). Aggressive fluid resuscitation initiated with 30 mL/kg crystalloid bolus. Despite 2 liters of IV normal saline, blood pressure remained 72/38 mmHg with MAP 49. Central venous catheter placed in the right internal jugular vein and norepinephrine infusion started at 0.15 mcg/kg/min, titrated to 0.3 mcg/kg/min to achieve MAP greater than 65 mmHg. Vasopressin 0.04 units/min added as a second vasopressor. Broad-spectrum antibiotics initiated: vancomycin 1.5 g IV, meropenem 1 g IV every 8 hours, and azithromycin 500 mg IV daily. Urgent automated red cell exchange transfusion performed, reducing HbS from 52% to 18%, with post-exchange hemoglobin of 9.8 g/dL.
+On ICU day 2, blood cultures returned positive for Streptococcus pneumoniae in both sets; antibiotics narrowed to ceftriaxone based on susceptibilities. Repeat ABG showed improvement: pH 7.31, PaCO2 34 mmHg, PaO2 72 mmHg on FiO2 80%. Serum creatinine peaked at 2.8 mg/dL on day 2 (2.8 times baseline of 1.0 mg/dL). Urine output improved to 0.5 mL/kg/hr after hemodynamic stabilization; renal replacement therapy was not required. By ICU day 4, vasopressors successfully weaned off and FiO2 reduced to 50%. Extubated on ICU day 6 to high-flow nasal cannula, then weaned to room air by day 8. Transferred to medical floor on day 7. Mental status returned to baseline. No seizures or focal neurological deficits observed throughout admission. No arrhythmias on continuous telemetry.
+DISCHARGE SUMMARY: Creatinine normalized to 1.1 mg/dL by discharge. Repeat chest X-ray showed near-complete resolution of bilateral infiltrates. No evidence of pulmonary embolism, stroke, or other neurological complications. Hearing intact bilaterally. PHQ-9 score 3 (minimal depression). Patient discharged on hospital day 14 in stable condition with close hematology follow-up.
+DISCHARGE DIAGNOSES: (1) Acute chest syndrome, life-threatening, requiring invasive mechanical ventilation and vasopressor support. (2) Acute sickle cell vaso-occlusive crisis complicated by acute chest syndrome and requiring life-supporting interventions. (3) Sepsis secondary to Streptococcus pneumoniae bacteremia with septic shock requiring vasopressor therapy. (4) Acute kidney injury, KDIGO stage 2, creatinine 2.8 times baseline, resolved without dialysis. (5) Fever, temperature 39.8 degrees Celsius.</t>
+        </is>
+      </c>
+      <c r="L20" s="10" t="inlineStr">
+        <is>
+          <t>5/22/96</t>
+        </is>
+      </c>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t>8/10/96</t>
+        </is>
+      </c>
+      <c r="N20" s="10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="O20" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P20" s="12" t="inlineStr"/>
+      <c r="Q20" s="12" t="inlineStr"/>
+      <c r="R20" s="12" t="inlineStr"/>
+      <c r="S20" s="12" t="inlineStr"/>
+      <c r="T20" s="12" t="inlineStr"/>
+      <c r="U20" s="12" t="inlineStr"/>
+      <c r="V20" s="12" t="inlineStr"/>
+      <c r="W20" s="12" t="inlineStr"/>
+      <c r="X20" s="12" t="inlineStr"/>
+      <c r="Y20" s="12" t="inlineStr"/>
+      <c r="Z20" s="12" t="inlineStr"/>
+      <c r="AA20" s="12" t="inlineStr"/>
+      <c r="AB20" s="12" t="inlineStr"/>
+      <c r="AC20" s="12" t="inlineStr"/>
+      <c r="AD20" s="12" t="inlineStr"/>
+      <c r="AE20" s="12" t="inlineStr"/>
+      <c r="AF20" s="12" t="inlineStr"/>
+      <c r="AG20" s="12" t="inlineStr"/>
+      <c r="AH20" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AI20" s="12" t="inlineStr"/>
+      <c r="AJ20" s="12" t="inlineStr"/>
+      <c r="AK20" s="12" t="inlineStr"/>
+      <c r="AL20" s="12" t="inlineStr"/>
+      <c r="AM20" s="12" t="inlineStr"/>
+      <c r="AN20" s="12" t="inlineStr"/>
+      <c r="AO20" s="12" t="inlineStr"/>
+      <c r="AP20" s="12" t="inlineStr"/>
+      <c r="AQ20" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AR20" s="12" t="inlineStr"/>
+      <c r="AS20" s="12" t="inlineStr"/>
+      <c r="AT20" s="12" t="inlineStr"/>
+      <c r="AU20" s="12" t="inlineStr"/>
+      <c r="AV20" s="12" t="inlineStr"/>
+      <c r="AW20" s="12" t="inlineStr"/>
+      <c r="AX20" s="12" t="inlineStr"/>
+      <c r="AY20" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AZ20" s="12" t="inlineStr"/>
+      <c r="BA20" s="12" t="inlineStr"/>
+      <c r="BB20" s="12" t="inlineStr"/>
+      <c r="BC20" s="12" t="inlineStr"/>
+      <c r="BD20" s="12" t="inlineStr"/>
+      <c r="BE20" s="12" t="inlineStr"/>
+      <c r="BF20" s="12" t="inlineStr"/>
+      <c r="BG20" s="12" t="inlineStr"/>
+      <c r="BH20" s="12" t="inlineStr"/>
+      <c r="BI20" s="12" t="inlineStr"/>
+      <c r="BJ20" s="12" t="inlineStr"/>
+      <c r="BK20" s="13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="BL20" s="12" t="inlineStr"/>
+      <c r="BM20" s="12" t="inlineStr"/>
+      <c r="BN20" s="12" t="inlineStr"/>
+      <c r="BO20" s="12" t="inlineStr"/>
+      <c r="BP20" s="12" t="inlineStr"/>
+    </row>
+    <row r="21" ht="200" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_004</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>5/2/25</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Telephone</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Back Pain</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>9.4</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>Warm</t>
+        </is>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>TELEPHONE ENCOUNTER NOTE
+PATIENT: 19-year-old female with sickle cell disease (HbSS), diagnosed at birth via newborn screening. Patient called the sickle cell clinic nurse line reporting onset of bilateral arm and back pain approximately 4 hours ago, rated 5 out of 10 in intensity. She states she has been taking her hydroxyurea as prescribed. She began her home pain management protocol consisting of oral hydromorphone 4 mg every 4 hours, ibuprofen 400 mg every 6 hours, oral hydration with at least 2 liters of fluids, and application of a heating pad to the affected areas. She reports her pain has decreased to 3 out of 10 after two doses of hydromorphone.
+She denies fever, chills, chest pain, shortness of breath, cough, abdominal pain, headache, vision changes, leg swelling, or urinary symptoms. She reports no recent illness or sick contacts. She denies any feelings of sadness, hopelessness, or loss of interest in activities. She states she is eating and drinking well. Her most recent clinic visit was 3 weeks ago with a PHQ-9 score of 3 (minimal symptoms, no treatment recommended). Baseline hemoglobin at last visit was 9.4 g/dL. Temperature at home measured 37.2 degrees Celsius (99.0 degrees Fahrenheit).
+ASSESSMENT: Mild acute sickle cell vaso-occlusive pain episode, well-controlled at home with oral analgesics and hydration. No signs or symptoms concerning for acute chest syndrome, fever, infection, or other complications. Patient is afebrile (37.2 degrees Celsius, below 38.0 threshold).
+PLAN: Continue home pain management protocol. Increase oral fluids. Rest with intermittent ambulation. Patient instructed to call back or present to the emergency department if pain worsens to 7 out of 10 or above, if she develops fever of 38.0 degrees Celsius or higher, chest pain, shortness of breath, or any new symptoms. Follow-up telephone call scheduled for tomorrow morning. Routine clinic appointment in 2 weeks.</t>
+        </is>
+      </c>
+      <c r="L21" s="10" t="inlineStr">
+        <is>
+          <t>8/14/05</t>
+        </is>
+      </c>
+      <c r="M21" s="10" t="inlineStr">
+        <is>
+          <t>8/17/05</t>
+        </is>
+      </c>
+      <c r="N21" s="10" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="O21" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P21" s="12" t="inlineStr"/>
+      <c r="Q21" s="12" t="inlineStr"/>
+      <c r="R21" s="12" t="inlineStr"/>
+      <c r="S21" s="12" t="inlineStr"/>
+      <c r="T21" s="12" t="inlineStr"/>
+      <c r="U21" s="12" t="inlineStr"/>
+      <c r="V21" s="12" t="inlineStr"/>
+      <c r="W21" s="12" t="inlineStr"/>
+      <c r="X21" s="12" t="inlineStr"/>
+      <c r="Y21" s="12" t="inlineStr"/>
+      <c r="Z21" s="12" t="inlineStr"/>
+      <c r="AA21" s="12" t="inlineStr"/>
+      <c r="AB21" s="12" t="inlineStr"/>
+      <c r="AC21" s="12" t="inlineStr"/>
+      <c r="AD21" s="12" t="inlineStr"/>
+      <c r="AE21" s="12" t="inlineStr"/>
+      <c r="AF21" s="12" t="inlineStr"/>
+      <c r="AG21" s="12" t="inlineStr"/>
+      <c r="AH21" s="12" t="inlineStr"/>
+      <c r="AI21" s="12" t="inlineStr"/>
+      <c r="AJ21" s="12" t="inlineStr"/>
+      <c r="AK21" s="12" t="inlineStr"/>
+      <c r="AL21" s="12" t="inlineStr"/>
+      <c r="AM21" s="12" t="inlineStr"/>
+      <c r="AN21" s="12" t="inlineStr"/>
+      <c r="AO21" s="12" t="inlineStr"/>
+      <c r="AP21" s="12" t="inlineStr"/>
+      <c r="AQ21" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AR21" s="12" t="inlineStr"/>
+      <c r="AS21" s="12" t="inlineStr"/>
+      <c r="AT21" s="12" t="inlineStr"/>
+      <c r="AU21" s="12" t="inlineStr"/>
+      <c r="AV21" s="12" t="inlineStr"/>
+      <c r="AW21" s="12" t="inlineStr"/>
+      <c r="AX21" s="12" t="inlineStr"/>
+      <c r="AY21" s="12" t="inlineStr"/>
+      <c r="AZ21" s="12" t="inlineStr"/>
+      <c r="BA21" s="12" t="inlineStr"/>
+      <c r="BB21" s="12" t="inlineStr"/>
+      <c r="BC21" s="12" t="inlineStr"/>
+      <c r="BD21" s="12" t="inlineStr"/>
+      <c r="BE21" s="12" t="inlineStr"/>
+      <c r="BF21" s="12" t="inlineStr"/>
+      <c r="BG21" s="12" t="inlineStr"/>
+      <c r="BH21" s="12" t="inlineStr"/>
+      <c r="BI21" s="12" t="inlineStr"/>
+      <c r="BJ21" s="12" t="inlineStr"/>
+      <c r="BK21" s="12" t="inlineStr"/>
+      <c r="BL21" s="12" t="inlineStr"/>
+      <c r="BM21" s="12" t="inlineStr"/>
+      <c r="BN21" s="12" t="inlineStr"/>
+      <c r="BO21" s="12" t="inlineStr"/>
+      <c r="BP21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22" ht="200" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_005</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>9/10/25</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Leg Pain</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 34-year-old male with sickle cell disease (HbSS) and a history of two prior vaso-occlusive crises requiring hospitalization in the past year presents to the emergency department with acute onset of severe right lower extremity pain and swelling that began yesterday. He describes deep, constant pain in his right calf and thigh rated 8 out of 10 in intensity, different from his usual sickle cell pain crises. He also reports bilateral hip and lower back pain consistent with his typical vaso-occlusive pain pattern, rated 7 out of 10. He denies fever, cough, shortness of breath, chest pain, hemoptysis, headache, vision changes, or abdominal pain. No history of prior DVT or pulmonary embolism. No recent surgery or prolonged immobilization.
+OBJECTIVE: Temperature 37.4 degrees Celsius (99.3 degrees Fahrenheit), heart rate 92 bpm, blood pressure 128/76 mmHg, respiratory rate 16 breaths/min, SpO2 97% on room air. General: Alert, oriented, in moderate distress from pain. HEENT: Mild scleral icterus. Lungs: Clear to auscultation bilaterally, no wheezes, crackles, or rhonchi. Cardiovascular: Regular rate and rhythm, no murmurs. Abdomen: Soft, non-tender, no hepatosplenomegaly. Right lower extremity: Notable swelling of the right calf (circumference 4 cm greater than left), warmth, erythema, and tenderness along the posterior calf. Positive Homans sign. Left lower extremity: No swelling, no tenderness. No leg ulcers bilaterally. Neurological: Alert and oriented x4, no focal deficits.
+LABS: Hemoglobin 8.1 g/dL (baseline 8.5 g/dL), WBC 9.8 x 10^3/uL, platelets 312 x 10^3/uL. D-dimer elevated at 2.4 mg/L. Serum creatinine 0.8 mg/dL (baseline 0.7 mg/dL). LDH 298 U/L, total bilirubin 2.8 mg/dL. Coagulation: INR 1.1, aPTT 28 seconds.
+IMAGING: Right lower extremity venous Doppler ultrasound: Non-compressible right popliteal vein with echogenic intraluminal thrombus extending into the distal superficial femoral vein, consistent with acute deep vein thrombosis. CT pulmonary angiography: No evidence of pulmonary embolism. No pulmonary infiltrates. Chest X-ray: Clear lungs, no infiltrates, no pleural effusions.
+HOSPITAL COURSE: Patient admitted to the medical floor for management of acute DVT and concurrent vaso-occlusive pain crisis. Heparin IV infusion initiated with anti-Xa level monitoring, transitioned to therapeutic enoxaparin 1 mg/kg subcutaneous every 12 hours on hospital day 2. No thrombolysis or surgical thrombectomy was required. The patient remained hemodynamically stable throughout admission with no signs of limb-threatening ischemia. Right leg swelling improved with elevation and anticoagulation. Pain managed with IV hydromorphone PCA, transitioned to oral analgesics on hospital day 3. No fever during admission (temperature remained below 38.0 degrees Celsius throughout). Repeat Doppler on day 3 showed stable thrombus without extension.
+DISCHARGE: Patient discharged on hospital day 4 in stable condition on rivaroxaban 15 mg twice daily for 21 days followed by 20 mg daily for DVT treatment. No evidence of pulmonary embolism, stroke, or ACS during admission. No arrhythmias on telemetry. Hearing intact. PHQ-9 not formally assessed this visit. Follow-up with hematology in 1 week and vascular medicine in 2 weeks.
+DISCHARGE DIAGNOSES: (1) Acute deep vein thrombosis, right popliteal and distal superficial femoral vein, managed with anticoagulation. (2) Acute sickle cell vaso-occlusive pain crisis requiring inpatient admission, without co-complications.</t>
+        </is>
+      </c>
+      <c r="L22" s="10" t="inlineStr">
+        <is>
+          <t>3/22/91</t>
+        </is>
+      </c>
+      <c r="M22" s="10" t="inlineStr">
+        <is>
+          <t>6/1/91</t>
+        </is>
+      </c>
+      <c r="N22" s="10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="O22" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P22" s="12" t="inlineStr"/>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R22" s="12" t="inlineStr"/>
+      <c r="S22" s="12" t="inlineStr"/>
+      <c r="T22" s="12" t="inlineStr"/>
+      <c r="U22" s="12" t="inlineStr"/>
+      <c r="V22" s="12" t="inlineStr"/>
+      <c r="W22" s="12" t="inlineStr"/>
+      <c r="X22" s="12" t="inlineStr"/>
+      <c r="Y22" s="12" t="inlineStr"/>
+      <c r="Z22" s="12" t="inlineStr"/>
+      <c r="AA22" s="12" t="inlineStr"/>
+      <c r="AB22" s="12" t="inlineStr"/>
+      <c r="AC22" s="12" t="inlineStr"/>
+      <c r="AD22" s="12" t="inlineStr"/>
+      <c r="AE22" s="12" t="inlineStr"/>
+      <c r="AF22" s="12" t="inlineStr"/>
+      <c r="AG22" s="12" t="inlineStr"/>
+      <c r="AH22" s="12" t="inlineStr"/>
+      <c r="AI22" s="12" t="inlineStr"/>
+      <c r="AJ22" s="12" t="inlineStr"/>
+      <c r="AK22" s="12" t="inlineStr"/>
+      <c r="AL22" s="12" t="inlineStr"/>
+      <c r="AM22" s="12" t="inlineStr"/>
+      <c r="AN22" s="12" t="inlineStr"/>
+      <c r="AO22" s="12" t="inlineStr"/>
+      <c r="AP22" s="12" t="inlineStr"/>
+      <c r="AQ22" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AR22" s="12" t="inlineStr"/>
+      <c r="AS22" s="12" t="inlineStr"/>
+      <c r="AT22" s="12" t="inlineStr"/>
+      <c r="AU22" s="12" t="inlineStr"/>
+      <c r="AV22" s="12" t="inlineStr"/>
+      <c r="AW22" s="12" t="inlineStr"/>
+      <c r="AX22" s="12" t="inlineStr"/>
+      <c r="AY22" s="12" t="inlineStr"/>
+      <c r="AZ22" s="12" t="inlineStr"/>
+      <c r="BA22" s="12" t="inlineStr"/>
+      <c r="BB22" s="12" t="inlineStr"/>
+      <c r="BC22" s="12" t="inlineStr"/>
+      <c r="BD22" s="12" t="inlineStr"/>
+      <c r="BE22" s="12" t="inlineStr"/>
+      <c r="BF22" s="12" t="inlineStr"/>
+      <c r="BG22" s="12" t="inlineStr"/>
+      <c r="BH22" s="12" t="inlineStr"/>
+      <c r="BI22" s="12" t="inlineStr"/>
+      <c r="BJ22" s="12" t="inlineStr"/>
+      <c r="BK22" s="12" t="inlineStr"/>
+      <c r="BL22" s="12" t="inlineStr"/>
+      <c r="BM22" s="12" t="inlineStr"/>
+      <c r="BN22" s="12" t="inlineStr"/>
+      <c r="BO22" s="12" t="inlineStr"/>
+      <c r="BP22" s="12" t="inlineStr"/>
+    </row>
+    <row r="23" ht="200" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_006</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>11/15/25</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Chest Pain</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>DEATH SUMMARY
+PATIENT: 42-year-old female with sickle cell disease (HbSS), history of recurrent acute chest syndrome (4 prior episodes), chronic kidney disease stage 3 (baseline eGFR 42 mL/min/1.73m2, baseline creatinine 1.8 mg/dL), systemic arterial hypertension on lisinopril, and iron overload secondary to chronic transfusion therapy.
+PRESENTATION: Patient presented to the emergency department via EMS with acute severe bilateral chest pain, dyspnea, and high-grade fever. Temperature 40.1 degrees Celsius (104.2 degrees Fahrenheit), heart rate 142 bpm, blood pressure 84/50 mmHg, respiratory rate 40 breaths/min, SpO2 68% on 15 L non-rebreather mask. Patient was in severe respiratory distress, obtunded with GCS 7 (E1 V2 M4).
+LABS ON ADMISSION: Hemoglobin 4.2 g/dL (baseline 7.5 g/dL), WBC 32.1 x 10^3/uL with 20% bands, platelets 42 x 10^3/uL. Serum creatinine 4.8 mg/dL (baseline 1.8 mg/dL, representing 2.67 times baseline). BUN 62 mg/dL. LDH 2,340 U/L. Total bilirubin 14.2 mg/dL. AST 312 U/L, ALT 178 U/L. Lactate 11.4 mmol/L. Procalcitonin 22.6 ng/mL. ABG: pH 7.08, PaCO2 22 mmHg, PaO2 38 mmHg on 15 L NRB. Troponin-T 0.89 ng/mL (elevated). INR 2.4, aPTT 58 seconds. Blood cultures: Two sets drawn.
+IMAGING: Chest X-ray: Dense bilateral multilobar consolidations involving all lung fields, bilateral pleural effusions. CT pulmonary angiography: No pulmonary embolism; confirmed diffuse bilateral airspace disease consistent with severe acute chest syndrome. No deep vein thrombosis on bilateral lower extremity Doppler.
+ICU COURSE: Patient emergently intubated in the ED for refractory hypoxemia and obtundation. Ventilator settings: FiO2 100%, PEEP 14 cmH2O. Despite maximal ventilatory support, PaO2 remained below 55 mmHg. Central venous access obtained. Norepinephrine infusion started and titrated to 0.8 mcg/kg/min. Vasopressin 0.04 units/min added. Epinephrine infusion added at 0.1 mcg/kg/min as a third vasopressor for refractory shock. Broad-spectrum antibiotics initiated. Emergency exchange transfusion attempted but was unable to be completed due to cardiovascular instability.
+On ICU day 1, blood cultures returned positive for Staphylococcus aureus in both sets. Creatinine rose to 5.6 mg/dL (3.11 times baseline) with urine output less than 10 mL/hr. Continuous renal replacement therapy (CRRT) initiated. Platelet count dropped to 28 x 10^3/uL. Patient developed refractory metabolic acidosis with pH 6.98 and lactate 18.2 mmol/L.
+On ICU day 2, patient developed pulseless electrical activity cardiac arrest. Advanced cardiac life support was performed for 45 minutes. Despite aggressive resuscitative efforts including epinephrine boluses, bicarbonate administration, and continued chest compressions, return of spontaneous circulation was not achieved.
+TIME OF DEATH: Pronounced dead at 14:32 on ICU day 2.
+CAUSE OF DEATH: Acute chest syndrome with refractory hypoxemic respiratory failure and multi-organ failure in the setting of sickle cell disease.
+FINAL DIAGNOSES:
+(1) Acute chest syndrome, fatal — death directly attributed to ACS with refractory respiratory failure.
+(2) Acute sickle cell vaso-occlusive crisis — death in the setting of acute pain episode.
+(3) Sepsis secondary to Staphylococcus aureus bacteremia.
+(4) Acute kidney injury, KDIGO stage 3 — creatinine 5.6 mg/dL (3.11 times baseline of 1.8 mg/dL), requiring continuous renal replacement therapy. Did not progress to ESRD.
+(5) Fever, temperature 40.1 degrees Celsius.
+(6) Acute multiorgan failure involving respiratory, renal, hepatic, and hematologic systems.</t>
+        </is>
+      </c>
+      <c r="L23" s="10" t="inlineStr">
+        <is>
+          <t>6/30/83</t>
+        </is>
+      </c>
+      <c r="M23" s="10" t="inlineStr">
+        <is>
+          <t>7/5/83</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="O23" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P23" s="12" t="inlineStr"/>
+      <c r="Q23" s="12" t="inlineStr"/>
+      <c r="R23" s="12" t="inlineStr"/>
+      <c r="S23" s="12" t="inlineStr"/>
+      <c r="T23" s="12" t="inlineStr"/>
+      <c r="U23" s="12" t="inlineStr"/>
+      <c r="V23" s="12" t="inlineStr"/>
+      <c r="W23" s="12" t="inlineStr"/>
+      <c r="X23" s="12" t="inlineStr"/>
+      <c r="Y23" s="12" t="inlineStr"/>
+      <c r="Z23" s="12" t="inlineStr"/>
+      <c r="AA23" s="12" t="inlineStr"/>
+      <c r="AB23" s="12" t="inlineStr"/>
+      <c r="AC23" s="12" t="inlineStr"/>
+      <c r="AD23" s="12" t="inlineStr"/>
+      <c r="AE23" s="12" t="inlineStr"/>
+      <c r="AF23" s="12" t="inlineStr"/>
+      <c r="AG23" s="12" t="inlineStr"/>
+      <c r="AH23" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AI23" s="12" t="inlineStr"/>
+      <c r="AJ23" s="12" t="inlineStr"/>
+      <c r="AK23" s="12" t="inlineStr"/>
+      <c r="AL23" s="12" t="inlineStr"/>
+      <c r="AM23" s="12" t="inlineStr"/>
+      <c r="AN23" s="12" t="inlineStr"/>
+      <c r="AO23" s="12" t="inlineStr"/>
+      <c r="AP23" s="12" t="inlineStr"/>
+      <c r="AQ23" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AR23" s="12" t="inlineStr"/>
+      <c r="AS23" s="12" t="inlineStr"/>
+      <c r="AT23" s="12" t="inlineStr"/>
+      <c r="AU23" s="12" t="inlineStr"/>
+      <c r="AV23" s="12" t="inlineStr"/>
+      <c r="AW23" s="12" t="inlineStr"/>
+      <c r="AX23" s="12" t="inlineStr"/>
+      <c r="AY23" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AZ23" s="12" t="inlineStr"/>
+      <c r="BA23" s="12" t="inlineStr"/>
+      <c r="BB23" s="12" t="inlineStr"/>
+      <c r="BC23" s="12" t="inlineStr"/>
+      <c r="BD23" s="12" t="inlineStr"/>
+      <c r="BE23" s="12" t="inlineStr"/>
+      <c r="BF23" s="12" t="inlineStr"/>
+      <c r="BG23" s="12" t="inlineStr"/>
+      <c r="BH23" s="12" t="inlineStr"/>
+      <c r="BI23" s="12" t="inlineStr"/>
+      <c r="BJ23" s="12" t="inlineStr"/>
+      <c r="BK23" s="13" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="BL23" s="12" t="inlineStr"/>
+      <c r="BM23" s="12" t="inlineStr"/>
+      <c r="BN23" s="12" t="inlineStr"/>
+      <c r="BO23" s="12" t="inlineStr"/>
+      <c r="BP23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24" ht="200" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_007</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>4/18/25</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Chest Pain</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>10.8</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>Mild</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 14-year-old female with sickle cell disease (HbSC), diagnosed at age 1, presents to the pediatric emergency department with right-sided chest pain and nonproductive cough that began this morning. She rates her chest pain at 4 out of 10. She also reports mild generalized body aches. Her mother states she had a runny nose and sore throat 3 days ago that has been improving. She denies high fever, shortness of breath, wheezing, abdominal pain, leg pain, leg swelling, headache, vision changes, or urinary symptoms. She is up to date on vaccinations. No history of prior ACS episodes. No depressive symptoms. Menses regular and normal.
+OBJECTIVE: Temperature 38.6 degrees Celsius (101.5 degrees Fahrenheit), heart rate 88 bpm, blood pressure 106/64 mmHg, respiratory rate 20 breaths/min, SpO2 97% on room air. General: Well-appearing adolescent, alert, in no acute distress. HEENT: Mild scleral icterus, oropharynx clear. Lungs: Diminished breath sounds at right lower lobe base, no wheezes or rhonchi. Scattered crackles at right base on deep inspiration. Cardiovascular: Regular rate and rhythm, no murmurs. Abdomen: Soft, non-tender, spleen not palpable. Extremities: No swelling, no tenderness, no leg ulcers. Full range of motion in all joints. Neurological: Alert and oriented, cranial nerves intact, no focal deficits.
+LABS: Hemoglobin 10.8 g/dL (baseline 11.2 g/dL), WBC 10.4 x 10^3/uL, platelets 245 x 10^3/uL, reticulocyte count 4.2%. Serum creatinine 0.5 mg/dL (baseline 0.5 mg/dL). LDH 210 U/L, total bilirubin 1.4 mg/dL.
+IMAGING: Chest X-ray: Small right lower lobe segmental opacity consistent with a new infiltrate. No pleural effusion. No other consolidation.
+ASSESSMENT: Mild acute chest syndrome — new right lower lobe infiltrate with cough and low-grade fever, with SpO2 97% on room air. The patient does not require supplemental oxygen, transfusion, erythropoietin, BiPAP, or any supportive treatment other than antibiotics. Concurrent mild pain episode treated in ED.
+PLAN: Started on oral azithromycin 500 mg day 1, then 250 mg daily for 4 days for community-acquired pneumonia coverage per ACS protocol. No supplemental oxygen needed (SpO2 97% on room air). No transfusion indicated given stable hemoglobin near baseline. Incentive spirometry instruction provided. Pain managed with oral ibuprofen 400 mg in the ED with improvement to 2 out of 10. Patient observed in ED for 5 hours with stable vital signs and oxygen saturation. Not admitted. Discharged home with oral antibiotics and pain medications. Mother instructed to return immediately if daughter develops worsening cough, fever above 39.0 degrees Celsius, shortness of breath, chest pain worsening, or oxygen saturations below 95% on home pulse oximeter. Follow-up with pediatric hematology in 24-48 hours.
+DISCHARGE DIAGNOSES: (1) Acute chest syndrome, mild, managed with antibiotics alone on room air without transfusion or respiratory support. (2) Acute sickle cell pain episode, treated in ED and discharged.</t>
+        </is>
+      </c>
+      <c r="L24" s="10" t="inlineStr">
+        <is>
+          <t>1/25/11</t>
+        </is>
+      </c>
+      <c r="M24" s="10" t="inlineStr">
+        <is>
+          <t>3/10/12</t>
+        </is>
+      </c>
+      <c r="N24" s="10" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="O24" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P24" s="12" t="inlineStr"/>
+      <c r="Q24" s="12" t="inlineStr"/>
+      <c r="R24" s="12" t="inlineStr"/>
+      <c r="S24" s="12" t="inlineStr"/>
+      <c r="T24" s="12" t="inlineStr"/>
+      <c r="U24" s="12" t="inlineStr"/>
+      <c r="V24" s="12" t="inlineStr"/>
+      <c r="W24" s="12" t="inlineStr"/>
+      <c r="X24" s="12" t="inlineStr"/>
+      <c r="Y24" s="12" t="inlineStr"/>
+      <c r="Z24" s="12" t="inlineStr"/>
+      <c r="AA24" s="12" t="inlineStr"/>
+      <c r="AB24" s="12" t="inlineStr"/>
+      <c r="AC24" s="12" t="inlineStr"/>
+      <c r="AD24" s="12" t="inlineStr"/>
+      <c r="AE24" s="12" t="inlineStr"/>
+      <c r="AF24" s="12" t="inlineStr"/>
+      <c r="AG24" s="12" t="inlineStr"/>
+      <c r="AH24" s="12" t="inlineStr"/>
+      <c r="AI24" s="12" t="inlineStr"/>
+      <c r="AJ24" s="12" t="inlineStr"/>
+      <c r="AK24" s="12" t="inlineStr"/>
+      <c r="AL24" s="12" t="inlineStr"/>
+      <c r="AM24" s="12" t="inlineStr"/>
+      <c r="AN24" s="12" t="inlineStr"/>
+      <c r="AO24" s="12" t="inlineStr"/>
+      <c r="AP24" s="12" t="inlineStr"/>
+      <c r="AQ24" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AR24" s="12" t="inlineStr"/>
+      <c r="AS24" s="12" t="inlineStr"/>
+      <c r="AT24" s="12" t="inlineStr"/>
+      <c r="AU24" s="12" t="inlineStr"/>
+      <c r="AV24" s="12" t="inlineStr"/>
+      <c r="AW24" s="12" t="inlineStr"/>
+      <c r="AX24" s="12" t="inlineStr"/>
+      <c r="AY24" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AZ24" s="12" t="inlineStr"/>
+      <c r="BA24" s="12" t="inlineStr"/>
+      <c r="BB24" s="12" t="inlineStr"/>
+      <c r="BC24" s="12" t="inlineStr"/>
+      <c r="BD24" s="12" t="inlineStr"/>
+      <c r="BE24" s="12" t="inlineStr"/>
+      <c r="BF24" s="12" t="inlineStr"/>
+      <c r="BG24" s="12" t="inlineStr"/>
+      <c r="BH24" s="12" t="inlineStr"/>
+      <c r="BI24" s="12" t="inlineStr"/>
+      <c r="BJ24" s="12" t="inlineStr"/>
+      <c r="BK24" s="13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BL24" s="12" t="inlineStr"/>
+      <c r="BM24" s="12" t="inlineStr"/>
+      <c r="BN24" s="12" t="inlineStr"/>
+      <c r="BO24" s="12" t="inlineStr"/>
+      <c r="BP24" s="12" t="inlineStr"/>
+    </row>
+    <row r="25" ht="200" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_008</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>6/5/25</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Pelvic Pain</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>7.6</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 16-year-old male with sickle cell disease (HbSS), presents to the pediatric emergency department with a painful, persistent penile erection that began approximately 5 hours ago. He reports the erection is fully rigid and extremely painful, rated 9 out of 10. He states he has had brief episodes of stuttering priapism (lasting less than 1 hour) approximately twice in the past 6 months, which resolved spontaneously. This episode has not resolved despite attempts at home remedies including warm compresses, ambulation, and oral pseudoephedrine 30 mg taken 3 hours ago. He also reports moderate bilateral thigh and lower back pain rated 6 out of 10, consistent with his typical vaso-occlusive pain pattern. He denies fever, cough, chest pain, shortness of breath, abdominal pain, headache, vision changes, or urinary difficulty prior to onset. No history of DVT, PE, or stroke.
+OBJECTIVE: Temperature 37.1 degrees Celsius (98.8 degrees Fahrenheit), heart rate 104 bpm, blood pressure 134/78 mmHg, respiratory rate 18 breaths/min, SpO2 99% on room air. General: Anxious adolescent male in significant distress. HEENT: Mild scleral icterus. Lungs: Clear to auscultation bilaterally. Cardiovascular: Tachycardic but regular rhythm, no murmurs. Abdomen: Soft, mildly tender in suprapubic region, no hepatosplenomegaly. Genitourinary: Fully rigid penile erection with tenderness of both corpora cavernosa. Glans is soft (not involved). No penile skin changes or necrosis. Extremities: Bilateral thigh tenderness, no swelling, no calf tenderness, no leg ulcers. Neurological: Alert and oriented, no focal deficits.
+LABS: Hemoglobin 7.6 g/dL (baseline 8.0 g/dL), WBC 12.1 x 10^3/uL, platelets 267 x 10^3/uL, reticulocyte count 11.3%. Serum creatinine 0.6 mg/dL (baseline 0.6 mg/dL). LDH 378 U/L, total bilirubin 3.4 mg/dL. Blood gas: Not obtained as patient is not in respiratory distress. Chest X-ray: Clear lungs, no infiltrates.
+EMERGENCY MANAGEMENT: Urology consulted emergently. Given duration greater than 4 hours and failure of conservative measures, the decision was made to proceed with corporal aspiration and irrigation. Under local penile block anesthesia (dorsal nerve block with 1% lidocaine without epinephrine), bilateral corporal aspiration was performed with 18-gauge butterfly needles. Approximately 60 mL of dark, deoxygenated blood was aspirated from each corpus cavernosum. Irrigation performed with dilute phenylephrine solution (100 mcg/mL in normal saline), injecting 1 mL aliquots every 3-5 minutes for a total of 5 injections per side. After the third irrigation cycle, progressive detumescence was observed. Full detumescence achieved within 30 minutes of initiating the procedure. No surgical shunt was required. Post-procedure examination confirmed a soft, non-tender phallus with normal color and perfusion.
+HOSPITAL COURSE: Patient admitted to the medical floor for observation and concurrent vaso-occlusive pain crisis management. IV normal saline initiated at maintenance rate. Pain managed with IV ketorolac 15 mg and IV morphine 0.1 mg/kg with adequate relief (pain reduced to 3 out of 10). Patient remained afebrile throughout (temperature maximum 37.4 degrees Celsius, never reaching 38.0 degrees Celsius). No recurrence of priapism during 24-hour observation period. No chest pain, cough, or respiratory symptoms developed. Repeat examination at 12 hours showed no recurrence.
+DISCHARGE: Patient discharged on hospital day 2 in stable condition. Started on daily oral pseudoephedrine 30 mg at bedtime for stuttering priapism prophylaxis. Pain controlled with oral analgesics. No evidence of ACS, stroke, DVT, PE, or fever during admission. Follow-up with pediatric hematology and urology in 1 week.
+DISCHARGE DIAGNOSES: (1) Ischemic priapism, 5-hour duration, treated with corporal aspiration and phenylephrine irrigation; no surgical shunt required. (2) Acute sickle cell vaso-occlusive pain crisis requiring inpatient admission, without co-complications.</t>
+        </is>
+      </c>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>12/10/08</t>
+        </is>
+      </c>
+      <c r="M25" s="10" t="inlineStr">
+        <is>
+          <t>12/15/08</t>
+        </is>
+      </c>
+      <c r="N25" s="10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="O25" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P25" s="12" t="inlineStr"/>
+      <c r="Q25" s="12" t="inlineStr"/>
+      <c r="R25" s="12" t="inlineStr"/>
+      <c r="S25" s="12" t="inlineStr"/>
+      <c r="T25" s="12" t="inlineStr"/>
+      <c r="U25" s="12" t="inlineStr"/>
+      <c r="V25" s="12" t="inlineStr"/>
+      <c r="W25" s="12" t="inlineStr"/>
+      <c r="X25" s="12" t="inlineStr"/>
+      <c r="Y25" s="12" t="inlineStr"/>
+      <c r="Z25" s="12" t="inlineStr"/>
+      <c r="AA25" s="12" t="inlineStr"/>
+      <c r="AB25" s="12" t="inlineStr"/>
+      <c r="AC25" s="12" t="inlineStr"/>
+      <c r="AD25" s="12" t="inlineStr"/>
+      <c r="AE25" s="12" t="inlineStr"/>
+      <c r="AF25" s="12" t="inlineStr"/>
+      <c r="AG25" s="12" t="inlineStr"/>
+      <c r="AH25" s="12" t="inlineStr"/>
+      <c r="AI25" s="12" t="inlineStr"/>
+      <c r="AJ25" s="12" t="inlineStr"/>
+      <c r="AK25" s="12" t="inlineStr"/>
+      <c r="AL25" s="12" t="inlineStr"/>
+      <c r="AM25" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AN25" s="12" t="inlineStr"/>
+      <c r="AO25" s="12" t="inlineStr"/>
+      <c r="AP25" s="12" t="inlineStr"/>
+      <c r="AQ25" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AR25" s="12" t="inlineStr"/>
+      <c r="AS25" s="12" t="inlineStr"/>
+      <c r="AT25" s="12" t="inlineStr"/>
+      <c r="AU25" s="12" t="inlineStr"/>
+      <c r="AV25" s="12" t="inlineStr"/>
+      <c r="AW25" s="12" t="inlineStr"/>
+      <c r="AX25" s="12" t="inlineStr"/>
+      <c r="AY25" s="12" t="inlineStr"/>
+      <c r="AZ25" s="12" t="inlineStr"/>
+      <c r="BA25" s="12" t="inlineStr"/>
+      <c r="BB25" s="12" t="inlineStr"/>
+      <c r="BC25" s="12" t="inlineStr"/>
+      <c r="BD25" s="12" t="inlineStr"/>
+      <c r="BE25" s="12" t="inlineStr"/>
+      <c r="BF25" s="12" t="inlineStr"/>
+      <c r="BG25" s="12" t="inlineStr"/>
+      <c r="BH25" s="12" t="inlineStr"/>
+      <c r="BI25" s="12" t="inlineStr"/>
+      <c r="BJ25" s="12" t="inlineStr"/>
+      <c r="BK25" s="12" t="inlineStr"/>
+      <c r="BL25" s="12" t="inlineStr"/>
+      <c r="BM25" s="12" t="inlineStr"/>
+      <c r="BN25" s="12" t="inlineStr"/>
+      <c r="BO25" s="12" t="inlineStr"/>
+      <c r="BP25" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A16:BP19"/>
+  <autoFilter ref="A17:BP25"/>
   <mergeCells count="14">
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
@@ -1625,7 +2366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1633,197 +2374,197 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>📋 ANSWER KEY — HOW TO USE THIS SHEET</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr"/>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>WHAT IS THIS?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>This sheet shows the ground-truth grading rationale for every outcome in each synthetic note.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Use it to verify that an AI extraction system (e.g., MedGemma) produces the correct grades.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>HOW TO READ EACH ROW</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>• Note ID — Which synthetic note (SYNTH_001, _002, or _003)</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>• Note ID — Which synthetic note (SYNTH_001 through SYNTH_008)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>• Outcome &amp; # — The SCOGS outcome name and its number (e.g., Fever = #36)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>• Grade — The correct ground-truth grade. Color-coded: green=1, yellow=2, orange=3, red=4, gray=absent</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>• Grade — The correct ground-truth grade. Color-coded: green=1, yellow=2, orange=3, red=4, dark red=5, gray=absent</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>• Feature Values — The exact clinical features extracted from the note that feed into the rule engine</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>• Rule Applied — The specific decision table rule from rules.md that produces this grade</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>• Key Quote — The verbatim text from the note that supports the feature extraction</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>HOW TO VERIFY A SYSTEM'S OUTPUT</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>1. Run the system on the note text from the 'Synthetic Notes' sheet</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>2. Compare its extracted features against the 'Feature Values' column below</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>3. Compare its assigned grade against the 'Grade' column — mismatches indicate extraction or grading errors</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>4. If the grade is wrong, check whether the system extracted the right quote (compare 'Key Quote' column)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Note ID</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Outcome</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Outcome #</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="14" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="14" t="inlineStr">
         <is>
           <t>Feature Values</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F21" s="14" t="inlineStr">
         <is>
           <t>Rule Applied</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
+      <c r="G21" s="14" t="inlineStr">
         <is>
           <t>Key Quote from Note</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
+    <row r="22" ht="55" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>SYNTH_001
 (Note 1)</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Acute Sickle Cell Pain Episode</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>care_setting = ed_treat_release
 pain_co_complication = false
@@ -1831,166 +2572,165 @@
 death_attributed = false</t>
         </is>
       </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>care_setting ≥ clinic AND care_setting &lt; inpatient → Grade 2</t>
-        </is>
-      </c>
-      <c r="G22" s="16" t="inlineStr">
-        <is>
-          <t>"Patient monitored in ED for 4 hours with improvement. Not admitted. Discharged home"</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ clinic AND &lt; inpatient → Grade 2</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>"Patient monitored in ED for 4 hours... Not admitted. Discharged home"</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="55" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>SYNTH_001
 (Note 1)</t>
         </is>
       </c>
-      <c r="B23" s="16" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Fever</t>
         </is>
       </c>
-      <c r="C23" s="16" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E23" s="16" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>temperature = 38.3 °C</t>
         </is>
       </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>38.0 ≤ temperature &lt; 38.5 → Grade 1</t>
-        </is>
-      </c>
-      <c r="G23" s="16" t="inlineStr">
-        <is>
-          <t>"Temperature 38.3 degrees Celsius (101.0 degrees Fahrenheit)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>38.0 ≤ temp &lt; 38.5 → Grade 1</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 38.3 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="55" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>SYNTH_001
 (Note 1)</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Acute Chest Syndrome</t>
         </is>
       </c>
-      <c r="C24" s="16" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>#48</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D24" s="18" t="inlineStr">
         <is>
           <t>absent</t>
         </is>
       </c>
-      <c r="E24" s="16" t="inlineStr">
-        <is>
-          <t>N/A — diagnostic criteria not met</t>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <t>No lobar infiltrate on imaging → absent</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>No lobar infiltrate</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>Diagnostic criteria not met → absent</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>"Chest X-ray: No acute cardiopulmonary disease, no infiltrates"</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="16" t="inlineStr"/>
-      <c r="B25" s="16" t="inlineStr"/>
-      <c r="C25" s="16" t="inlineStr"/>
-      <c r="D25" s="16" t="inlineStr"/>
-      <c r="E25" s="16" t="inlineStr"/>
-      <c r="F25" s="16" t="inlineStr"/>
-      <c r="G25" s="16" t="inlineStr"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
+    <row r="25" ht="55" customHeight="1">
+      <c r="A25" s="15" t="inlineStr"/>
+      <c r="B25" s="15" t="inlineStr"/>
+      <c r="C25" s="15" t="inlineStr"/>
+      <c r="D25" s="15" t="inlineStr"/>
+      <c r="E25" s="15" t="inlineStr"/>
+      <c r="F25" s="15" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr"/>
+    </row>
+    <row r="26" ht="55" customHeight="1">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Acute Sickle Cell Pain Episode</t>
         </is>
       </c>
-      <c r="C26" s="16" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>care_setting = inpatient
 pain_co_complication = true
-life_support = false
-death_attributed = false</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>pain_co_complication = true → Grade 4</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
-          <t>"Acute sickle cell vaso-occlusive pain crisis complicated by acute chest syndrome"</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+life_support = false</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>pain_co_complication → Grade 4</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>"pain crisis complicated by acute chest syndrome"</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="55" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Acute Chest Syndrome</t>
         </is>
       </c>
-      <c r="C27" s="16" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>#48</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D27" s="20" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>fio2_pct = 60%
 resp_support = high_flow
@@ -1998,167 +2738,126 @@
 life_support = false</t>
         </is>
       </c>
-      <c r="F27" s="16" t="inlineStr">
-        <is>
-          <t>(fio2 ≥ 50 OR resp_support ≥ high_flow OR exchange) AND NOT life_support → Grade 3</t>
-        </is>
-      </c>
-      <c r="G27" s="16" t="inlineStr">
-        <is>
-          <t>"high-flow nasal cannula at 40 L/min with FiO2 60%"; "Automated red cell exchange performed"</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="60" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
+        <is>
+          <t>(fio2≥50 OR high_flow OR exchange) AND NOT life_support → Grade 3</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>"high-flow nasal cannula at 40 L/min with FiO2 60%"; "red cell exchange performed"</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="55" customHeight="1">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>SYNTH_002
 (Note 2)</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Fever</t>
         </is>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
       </c>
-      <c r="D28" s="17" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>temperature = 39.2 °C</t>
         </is>
       </c>
-      <c r="F28" s="16" t="inlineStr">
-        <is>
-          <t>temperature ≥ 38.5 → Grade 2</t>
-        </is>
-      </c>
-      <c r="G28" s="16" t="inlineStr">
-        <is>
-          <t>"Temperature 39.2 degrees Celsius (102.6 degrees Fahrenheit)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1">
-      <c r="A29" s="16" t="inlineStr">
-        <is>
-          <t>SYNTH_002
-(Note 2)</t>
-        </is>
-      </c>
-      <c r="B29" s="16" t="inlineStr">
-        <is>
-          <t>AKI</t>
-        </is>
-      </c>
-      <c r="C29" s="16" t="inlineStr">
-        <is>
-          <t>#19</t>
-        </is>
-      </c>
-      <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>absent</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>creatinine_x_baseline = 1.13
-(below 1.5 threshold)</t>
-        </is>
-      </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>creatinine_x_baseline &lt; 1.5 → absent</t>
-        </is>
-      </c>
-      <c r="G29" s="16" t="inlineStr">
-        <is>
-          <t>"Serum creatinine 0.9 mg/dL (baseline 0.8 mg/dL, ratio 1.13x baseline)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="60" customHeight="1">
-      <c r="A30" s="16" t="inlineStr"/>
-      <c r="B30" s="16" t="inlineStr"/>
-      <c r="C30" s="16" t="inlineStr"/>
-      <c r="D30" s="16" t="inlineStr"/>
-      <c r="E30" s="16" t="inlineStr"/>
-      <c r="F30" s="16" t="inlineStr"/>
-      <c r="G30" s="16" t="inlineStr"/>
-    </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
+        <is>
+          <t>temp ≥ 38.5 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 39.2 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="55" customHeight="1">
+      <c r="A29" s="15" t="inlineStr"/>
+      <c r="B29" s="15" t="inlineStr"/>
+      <c r="C29" s="15" t="inlineStr"/>
+      <c r="D29" s="15" t="inlineStr"/>
+      <c r="E29" s="15" t="inlineStr"/>
+      <c r="F29" s="15" t="inlineStr"/>
+      <c r="G29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30" ht="55" customHeight="1">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Acute Sickle Cell Pain Episode</t>
         </is>
       </c>
-      <c r="C31" s="16" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>#28</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E31" s="16" t="inlineStr">
-        <is>
-          <t>care_setting = icu
-pain_co_complication = true
-life_support = true
-death_attributed = false</t>
-        </is>
-      </c>
-      <c r="F31" s="16" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t>pain_co_complication = true
+life_support = true</t>
+        </is>
+      </c>
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>pain_co_complication OR life_support → Grade 4</t>
         </is>
       </c>
-      <c r="G31" s="16" t="inlineStr">
-        <is>
-          <t>"vaso-occlusive crisis complicated by acute chest syndrome and requiring life-supporting interventions"</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="60" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>"crisis complicated by ACS and requiring life-supporting interventions"</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="55" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Acute Chest Syndrome</t>
         </is>
       </c>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>#48</t>
         </is>
       </c>
-      <c r="D32" s="20" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E32" s="16" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>fio2_pct = 100%
 resp_support = invasive_ventilation
@@ -2166,225 +2865,880 @@
 life_support = true</t>
         </is>
       </c>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>(fio2 ≥ 50 OR resp_support ≥ high_flow OR exchange) AND life_support → Grade 4</t>
-        </is>
-      </c>
-      <c r="G32" s="16" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
+        <is>
+          <t>(fio2≥50 OR high_flow OR exchange) AND life_support → Grade 4</t>
+        </is>
+      </c>
+      <c r="G31" s="15" t="inlineStr">
         <is>
           <t>"FiO2 100%"; "emergently intubated"; "norepinephrine"; "vasopressin"</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="60" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
+    <row r="32" ht="55" customHeight="1">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Fever</t>
         </is>
       </c>
-      <c r="C33" s="16" t="inlineStr">
+      <c r="C32" s="15" t="inlineStr">
         <is>
           <t>#36</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
+      <c r="D32" s="16" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E33" s="16" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>temperature = 39.8 °C</t>
         </is>
       </c>
-      <c r="F33" s="16" t="inlineStr">
-        <is>
-          <t>temperature ≥ 38.5 → Grade 2</t>
-        </is>
-      </c>
-      <c r="G33" s="16" t="inlineStr">
-        <is>
-          <t>"Temperature 39.8 degrees Celsius (103.6 degrees Fahrenheit)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="F32" s="15" t="inlineStr">
+        <is>
+          <t>temp ≥ 38.5 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 39.8 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="55" customHeight="1">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>SYNTH_003
 (Note 3)</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>Acute Kidney Injury</t>
         </is>
       </c>
-      <c r="C34" s="16" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>#19</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E34" s="16" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>creatinine_x_baseline = 2.8
-creatinine = 2.8 mg/dL
-renal_replacement = false
+renal_replacement = false</t>
+        </is>
+      </c>
+      <c r="F33" s="15" t="inlineStr">
+        <is>
+          <t>2.0 ≤ creatinine_x_baseline ≤ 2.9 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>"creatinine peaked at 2.8 mg/dL (2.8 times baseline of 1.0)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="55" customHeight="1">
+      <c r="A34" s="15" t="inlineStr"/>
+      <c r="B34" s="15" t="inlineStr"/>
+      <c r="C34" s="15" t="inlineStr"/>
+      <c r="D34" s="15" t="inlineStr"/>
+      <c r="E34" s="15" t="inlineStr"/>
+      <c r="F34" s="15" t="inlineStr"/>
+      <c r="G34" s="15" t="inlineStr"/>
+    </row>
+    <row r="35" ht="55" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_004
+(Note 4)</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = home
+pain_co_complication = false
+life_support = false</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>care_setting == home → Grade 1</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>"Patient called the sickle cell clinic nurse line"; managed at home with oral analgesics</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="55" customHeight="1">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_004
+(Note 4)</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D36" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>temperature = 37.2 °C</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>temp &lt; 38.0 → absent</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature at home measured 37.2 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="55" customHeight="1">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_004
+(Note 4)</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>Depression</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>#47</t>
+        </is>
+      </c>
+      <c r="D37" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>PHQ-9 = 3
+treatment_recommended = false</t>
+        </is>
+      </c>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>PHQ-9 &lt; 5 → absent</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>"PHQ-9 score of 3 (minimal symptoms, no treatment recommended)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="55" customHeight="1">
+      <c r="A38" s="15" t="inlineStr"/>
+      <c r="B38" s="15" t="inlineStr"/>
+      <c r="C38" s="15" t="inlineStr"/>
+      <c r="D38" s="15" t="inlineStr"/>
+      <c r="E38" s="15" t="inlineStr"/>
+      <c r="F38" s="15" t="inlineStr"/>
+      <c r="G38" s="15" t="inlineStr"/>
+    </row>
+    <row r="39" ht="55" customHeight="1">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_005
+(Note 5)</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = inpatient
+pain_co_complication = false
+life_support = false</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ inpatient AND NOT co_complication → Grade 3</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>"admitted to the medical floor"; "without co-complications"</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="55" customHeight="1">
+      <c r="A40" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_005
+(Note 5)</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>Deep Vein Thrombosis</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>#02</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>anticoagulation = true
+thrombolysis = false
+surgical_thrombectomy = false</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>anticoagulation AND NOT thrombolysis/surgery → Grade 2</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>"Heparin IV infusion initiated"; "No thrombolysis or surgical thrombectomy"</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="55" customHeight="1">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_005
+(Note 5)</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D41" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>temperature &lt; 38.0 °C throughout</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>temp &lt; 38.0 → absent</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>"temperature remained below 38.0 degrees Celsius throughout"</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="55" customHeight="1">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_005
+(Note 5)</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>Pulmonary Embolism</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>#51</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>Negative CTPA</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>No PE on imaging → absent</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>"CT pulmonary angiography: No evidence of pulmonary embolism"</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="55" customHeight="1">
+      <c r="A43" s="15" t="inlineStr"/>
+      <c r="B43" s="15" t="inlineStr"/>
+      <c r="C43" s="15" t="inlineStr"/>
+      <c r="D43" s="15" t="inlineStr"/>
+      <c r="E43" s="15" t="inlineStr"/>
+      <c r="F43" s="15" t="inlineStr"/>
+      <c r="G43" s="15" t="inlineStr"/>
+    </row>
+    <row r="44" ht="55" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_006
+(Note 6)</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>Acute Chest Syndrome</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="D44" s="21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>death_attributed = true</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>death_attributed → Grade 5</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>"Acute chest syndrome, fatal — death directly attributed to ACS"</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="55" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_006
+(Note 6)</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>death_attributed = true</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>death_attributed → Grade 5</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>"death in the setting of acute pain episode"</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="55" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_006
+(Note 6)</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>Acute Kidney Injury</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>#19</t>
+        </is>
+      </c>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>creatinine_x_baseline = 3.11
+creatinine = 5.6 mg/dL
+renal_replacement = true (CRRT)
 esrd_progression = false</t>
         </is>
       </c>
-      <c r="F34" s="16" t="inlineStr">
-        <is>
-          <t>2.0 ≤ creatinine_x_baseline ≤ 2.9 → Grade 2</t>
-        </is>
-      </c>
-      <c r="G34" s="16" t="inlineStr">
-        <is>
-          <t>"creatinine peaked at 2.8 mg/dL on day 2 (2.8 times baseline of 1.0 mg/dL)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="60" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>SYNTH_003
-(Note 3)</t>
-        </is>
-      </c>
-      <c r="B35" s="16" t="inlineStr">
-        <is>
-          <t>Sepsis</t>
-        </is>
-      </c>
-      <c r="C35" s="16" t="inlineStr">
-        <is>
-          <t>#37</t>
-        </is>
-      </c>
-      <c r="D35" s="22" t="inlineStr">
-        <is>
-          <t>present*</t>
-        </is>
-      </c>
-      <c r="E35" s="16" t="inlineStr">
-        <is>
-          <t>Positive blood cultures (S. pneumoniae)
-Vasopressor requirement
-*Grade requires rules.md §37</t>
-        </is>
-      </c>
-      <c r="F35" s="16" t="inlineStr">
-        <is>
-          <t>Clinically evident; exact SCOGS grade requires team verification per rules.md §37</t>
-        </is>
-      </c>
-      <c r="G35" s="16" t="inlineStr">
-        <is>
-          <t>"blood cultures returned positive for Streptococcus pneumoniae"; "norepinephrine"; "vasopressin"</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="23" t="inlineStr">
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>(creat_x_base ≥ 3.0 OR creat ≥ 4 OR RRT) AND NOT esrd → Grade 3</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>"Creatinine rose to 5.6 mg/dL (3.11 times baseline)"; "CRRT initiated"</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="55" customHeight="1">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_006
+(Note 6)</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>temperature = 40.1 °C</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>temp ≥ 38.5 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 40.1 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="55" customHeight="1">
+      <c r="A48" s="15" t="inlineStr"/>
+      <c r="B48" s="15" t="inlineStr"/>
+      <c r="C48" s="15" t="inlineStr"/>
+      <c r="D48" s="15" t="inlineStr"/>
+      <c r="E48" s="15" t="inlineStr"/>
+      <c r="F48" s="15" t="inlineStr"/>
+      <c r="G48" s="15" t="inlineStr"/>
+    </row>
+    <row r="49" ht="55" customHeight="1">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_007
+(Note 7)</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>Acute Chest Syndrome</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>resp_support = room_air
+transfusion_type = none
+acs_other_support = false
+fio2_pct = 21%</t>
+        </is>
+      </c>
+      <c r="F49" s="15" t="inlineStr">
+        <is>
+          <t>room_air AND no transfusion AND no other support → Grade 1</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr">
+        <is>
+          <t>"managed with antibiotics alone on room air without transfusion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="55" customHeight="1">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_007
+(Note 7)</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = ed_treat_release
+pain_co_complication = false</t>
+        </is>
+      </c>
+      <c r="F50" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ clinic AND &lt; inpatient → Grade 2</t>
+        </is>
+      </c>
+      <c r="G50" s="15" t="inlineStr">
+        <is>
+          <t>"observed in ED for 5 hours... Not admitted. Discharged home"</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="55" customHeight="1">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_007
+(Note 7)</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>temperature = 38.6 °C</t>
+        </is>
+      </c>
+      <c r="F51" s="15" t="inlineStr">
+        <is>
+          <t>temp ≥ 38.5 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G51" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 38.6 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="55" customHeight="1">
+      <c r="A52" s="15" t="inlineStr"/>
+      <c r="B52" s="15" t="inlineStr"/>
+      <c r="C52" s="15" t="inlineStr"/>
+      <c r="D52" s="15" t="inlineStr"/>
+      <c r="E52" s="15" t="inlineStr"/>
+      <c r="F52" s="15" t="inlineStr"/>
+      <c r="G52" s="15" t="inlineStr"/>
+    </row>
+    <row r="53" ht="55" customHeight="1">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_008
+(Note 8)</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>Priapism</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>#24</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E53" s="15" t="inlineStr">
+        <is>
+          <t>priapism_intervention = aspiration_irrigation</t>
+        </is>
+      </c>
+      <c r="F53" s="15" t="inlineStr">
+        <is>
+          <t>aspiration_irrigation → Grade 3</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="inlineStr">
+        <is>
+          <t>"corporal aspiration was performed"; "Irrigation with phenylephrine"; no shunt</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="55" customHeight="1">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_008
+(Note 8)</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E54" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = inpatient
+pain_co_complication = false</t>
+        </is>
+      </c>
+      <c r="F54" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ inpatient AND NOT co_complication → Grade 3</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>"admitted to the medical floor"; "without co-complications"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="55" customHeight="1">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_008
+(Note 8)</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>temperature max 37.4 °C</t>
+        </is>
+      </c>
+      <c r="F55" s="15" t="inlineStr">
+        <is>
+          <t>temp &lt; 38.0 → absent</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>"afebrile throughout (temperature maximum 37.4 degrees Celsius)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Grade Legend:</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="24" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="23" t="inlineStr">
         <is>
           <t>Grade 1 — Mild</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="25" t="inlineStr">
+      <c r="B59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="24" t="inlineStr">
         <is>
           <t>Grade 2 — Moderate</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="26" t="inlineStr">
+      <c r="B60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
         <is>
           <t>Grade 3 — Severe</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="27" t="inlineStr">
+      <c r="B61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="26" t="inlineStr">
         <is>
           <t>Grade 4 — Life-Threatening</t>
         </is>
       </c>
-      <c r="B42" s="6" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="28" t="inlineStr">
-        <is>
-          <t>Grade 5 — Fatal (not used in current notes)</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="29" t="inlineStr">
+      <c r="B62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="27" t="inlineStr">
+        <is>
+          <t>Grade 5 — Fatal</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr">
         <is>
           <t>Absent — Outcome not present</t>
         </is>
       </c>
-      <c r="B44" s="6" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>Present* — Needs team verification</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="n"/>
+      <c r="B64" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="24">
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A64:B64"/>
     <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A60:B60"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A45:B45"/>
     <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A61:B61"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A41:B41"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A11:G11"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A6:G6"/>
-    <mergeCell ref="A42:B42"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A62:B62"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A43:B43"/>
     <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A12:G12"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 4 new synthetic notes (SYNTH_009-012) addressing critical gaps
New notes expand coverage and test system precision:
- Note 9 (SYNTH_009): Grade 2 ACS (moderate) — completes ACS grades 1-5
- Note 10 (SYNTH_010): Grade 3 Stroke — first CNS outcome
- Note 11 (SYNTH_011): Grade 3 Sepsis — first pediatric patient <10 yrs, first sepsis grade
- Note 12 (SYNTH_012): Borderline edge cases — tests system precision by presenting values just below grading thresholds (Fever, AKI, ACS, DVT, Depression)

Updated CSV (12 rows), answer key markdown, and Excel workbook with all entries.
</commit_message>
<xml_diff>
--- a/data/synthetic_notes.xlsx
+++ b/data/synthetic_notes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Answer Key" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthetic Notes'!$A$17:$BP$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthetic Notes'!$A$17:$BP$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP25"/>
+  <dimension ref="A1:BP29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2338,8 +2338,585 @@
       <c r="BO25" s="12" t="inlineStr"/>
       <c r="BP25" s="12" t="inlineStr"/>
     </row>
+    <row r="26" ht="200" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_009</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>8/12/25</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Chest Pain</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 25-year-old male with sickle cell disease (HbSS) presents to the emergency department with acute onset of left-sided pleuritic chest pain, nonproductive cough, and subjective fevers since last night. He rates his chest pain at 6 out of 10, worsening with deep inspiration. He also reports diffuse body aches rated 5 out of 10, consistent with his typical pain crisis pattern. He denies hemoptysis, leg swelling, headache, visual changes, or abdominal pain. He has had one prior episode of acute chest syndrome two years ago that resolved with antibiotics and supplemental oxygen. No prior DVT or PE. No history of stroke.
+OBJECTIVE: Temperature 39.0 degrees Celsius (102.2 degrees Fahrenheit), heart rate 102 bpm, blood pressure 118/72 mmHg, respiratory rate 24 breaths/min, SpO2 91% on room air. General: Mildly ill-appearing, alert, oriented, speaking in full sentences. HEENT: Scleral icterus. Lungs: Decreased breath sounds at left lower lobe with dullness to percussion and scattered crackles. Right lung clear. Cardiovascular: Tachycardic, regular rhythm, no murmurs. Abdomen: Soft, non-tender, no hepatosplenomegaly. Extremities: No swelling, no tenderness, no calf tenderness, no leg ulcers. Neurological: Alert and oriented x4, no focal deficits.
+LABS: Hemoglobin 7.0 g/dL (baseline 8.8 g/dL, drop of 1.8 g/dL), WBC 14.2 x 10^3/uL, platelets 210 x 10^3/uL, reticulocyte count 9.8%. HbS 72%. Serum creatinine 0.9 mg/dL (baseline 0.9 mg/dL). LDH 445 U/L, total bilirubin 4.1 mg/dL. ABG: pH 7.41, PaCO2 36 mmHg, PaO2 64 mmHg on room air. Blood cultures obtained. CT pulmonary angiography: No pulmonary embolism. New left lower lobe consolidation consistent with acute chest syndrome. No pleural effusion.
+HOSPITAL COURSE: Patient admitted to the medical floor. Initiated on ceftriaxone and azithromycin for ACS coverage. Supplemental oxygen started via nasal cannula at 2 L/min (FiO2 approximately 28%), improving SpO2 to 95%. Given the 1.8 g/dL hemoglobin drop below baseline and ongoing oxygen requirement, hematology recommended a simple red blood cell transfusion. Patient received 2 units of packed red blood cells, with post-transfusion hemoglobin of 9.1 g/dL. No exchange transfusion was performed. Patient did not require high-flow nasal cannula, BiPAP, or any form of non-invasive or invasive ventilation. No vasopressors or other life-support interventions were needed. No erythropoietin was given. Pain managed with IV ketorolac and oral oxycodone with adequate relief.
+Patient improved steadily. Weaned to room air on hospital day 3 with SpO2 96%. Temperature normalized by day 2. Blood cultures returned negative. No arrhythmias on telemetry. No neurological complications. Repeat chest X-ray showed improving left lower lobe opacity.
+DISCHARGE: Discharged on hospital day 4 in stable condition. Follow-up in 1 week.
+DISCHARGE DIAGNOSES: (1) Acute chest syndrome, moderate, requiring low-flow supplemental oxygen (FiO2 28%) and simple erythrocyte transfusion; no exchange transfusion, no high-flow oxygen, no BiPAP, no ventilatory support. (2) Acute sickle cell vaso-occlusive pain crisis requiring inpatient admission without co-complications. (3) Fever, temperature 39.0 degrees Celsius.</t>
+        </is>
+      </c>
+      <c r="L26" s="10" t="inlineStr">
+        <is>
+          <t>2/18/00</t>
+        </is>
+      </c>
+      <c r="M26" s="10" t="inlineStr">
+        <is>
+          <t>5/1/00</t>
+        </is>
+      </c>
+      <c r="N26" s="10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="O26" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr"/>
+      <c r="Q26" s="12" t="inlineStr"/>
+      <c r="R26" s="12" t="inlineStr"/>
+      <c r="S26" s="12" t="inlineStr"/>
+      <c r="T26" s="12" t="inlineStr"/>
+      <c r="U26" s="12" t="inlineStr"/>
+      <c r="V26" s="12" t="inlineStr"/>
+      <c r="W26" s="12" t="inlineStr"/>
+      <c r="X26" s="12" t="inlineStr"/>
+      <c r="Y26" s="12" t="inlineStr"/>
+      <c r="Z26" s="12" t="inlineStr"/>
+      <c r="AA26" s="12" t="inlineStr"/>
+      <c r="AB26" s="12" t="inlineStr"/>
+      <c r="AC26" s="12" t="inlineStr"/>
+      <c r="AD26" s="12" t="inlineStr"/>
+      <c r="AE26" s="12" t="inlineStr"/>
+      <c r="AF26" s="12" t="inlineStr"/>
+      <c r="AG26" s="12" t="inlineStr"/>
+      <c r="AH26" s="12" t="inlineStr"/>
+      <c r="AI26" s="12" t="inlineStr"/>
+      <c r="AJ26" s="12" t="inlineStr"/>
+      <c r="AK26" s="12" t="inlineStr"/>
+      <c r="AL26" s="12" t="inlineStr"/>
+      <c r="AM26" s="12" t="inlineStr"/>
+      <c r="AN26" s="12" t="inlineStr"/>
+      <c r="AO26" s="12" t="inlineStr"/>
+      <c r="AP26" s="12" t="inlineStr"/>
+      <c r="AQ26" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AR26" s="12" t="inlineStr"/>
+      <c r="AS26" s="12" t="inlineStr"/>
+      <c r="AT26" s="12" t="inlineStr"/>
+      <c r="AU26" s="12" t="inlineStr"/>
+      <c r="AV26" s="12" t="inlineStr"/>
+      <c r="AW26" s="12" t="inlineStr"/>
+      <c r="AX26" s="12" t="inlineStr"/>
+      <c r="AY26" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AZ26" s="12" t="inlineStr"/>
+      <c r="BA26" s="12" t="inlineStr"/>
+      <c r="BB26" s="12" t="inlineStr"/>
+      <c r="BC26" s="12" t="inlineStr"/>
+      <c r="BD26" s="12" t="inlineStr"/>
+      <c r="BE26" s="12" t="inlineStr"/>
+      <c r="BF26" s="12" t="inlineStr"/>
+      <c r="BG26" s="12" t="inlineStr"/>
+      <c r="BH26" s="12" t="inlineStr"/>
+      <c r="BI26" s="12" t="inlineStr"/>
+      <c r="BJ26" s="12" t="inlineStr"/>
+      <c r="BK26" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="BL26" s="12" t="inlineStr"/>
+      <c r="BM26" s="12" t="inlineStr"/>
+      <c r="BN26" s="12" t="inlineStr"/>
+      <c r="BO26" s="12" t="inlineStr"/>
+      <c r="BP26" s="12" t="inlineStr"/>
+    </row>
+    <row r="27" ht="200" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_010</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>10/3/25</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>Cool</t>
+        </is>
+      </c>
+      <c r="K27" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 31-year-old female with sickle cell disease (HbSS), history of elevated TCD velocities in childhood treated with chronic transfusion therapy (discontinued at age 18), presents to the emergency department brought by her partner after acute onset of right-sided weakness and slurred speech approximately 2 hours ago. She was in her usual state of health prior to the event and denies any preceding headache, fever, chest pain, or pain crisis symptoms. She has no prior history of stroke or transient ischemic attack. She denies recent illness. Current medications: hydroxyurea 1000 mg daily, folic acid.
+OBJECTIVE: Temperature 37.0 degrees Celsius (98.6 degrees Fahrenheit), heart rate 88 bpm, blood pressure 142/86 mmHg, respiratory rate 16 breaths/min, SpO2 98% on room air. General: Alert, anxious, able to follow commands but with difficulty speaking. HEENT: Mild scleral icterus. No carotid bruits. Lungs: Clear to auscultation bilaterally. Cardiovascular: Regular rate and rhythm, grade I/VI systolic murmur. Abdomen: Soft, non-tender. Neurological examination: NIHSS score 8 at presentation. Right facial droop (central pattern, lower face). Dysarthria — moderate, slurred but intelligible speech. Right upper extremity: 3/5 strength with pronator drift. Right lower extremity: 4/5 strength. Left upper and lower extremities: 5/5 strength. Sensation intact bilaterally. Visual fields full to confrontation. No neglect. No leg ulcers.
+LABS: Hemoglobin 8.6 g/dL (baseline 9.0 g/dL), WBC 8.9 x 10^3/uL, platelets 340 x 10^3/uL. HbS 68%. Serum creatinine 0.7 mg/dL (baseline 0.7 mg/dL). Coagulation: INR 1.0, aPTT 28 seconds. Glucose 104 mg/dL.
+IMAGING: CT head without contrast (emergent): No acute hemorrhage. Early loss of gray-white differentiation in left MCA territory. CT angiography: Narrowing of the left middle cerebral artery M1 segment, no complete occlusion. MRI brain (obtained within 4 hours): Acute ischemic infarct in the left middle cerebral artery territory involving the left frontal and parietal cortex, confirmed on DWI and ADC sequences. No hemorrhagic transformation. Chest X-ray: No infiltrates, no acute cardiopulmonary process.
+HOSPITAL COURSE: Neurology and hematology consulted emergently. Given the acute ischemic stroke in the setting of SCD, IV tPA was not administered per institutional protocol (relative contraindication with SCD). Urgent exchange transfusion initiated within 3 hours of symptom onset, reducing HbS from 68% to 22%. Patient admitted to the neurological ICU for close monitoring. Aspirin 81 mg daily started. Blood pressure managed with permissive hypertension protocol (target SBP &lt; 180). No vasopressors or life-support interventions required. Patient was hemodynamically stable and breathing independently on room air throughout the ICU stay.
+Over hospital days 2 through 5, right-sided weakness partially improved. Right upper extremity strength improved from 3/5 to 4/5, right lower extremity to 4+/5. Dysarthria improved but persisted with mild slurring. Facial droop improved. Speech therapy and physical therapy initiated. Patient was able to ambulate with a cane by day 5. Transferred to medical floor on day 3. No fever throughout admission (temperature remained below 38.0 degrees Celsius). No chest pain or respiratory symptoms — no evidence of ACS. Blood cultures not obtained (no infectious indication). No arrhythmias on telemetry.
+DISCHARGE: Modified Rankin Scale (mRS) at discharge: 2 — slight disability, unable to carry out all previous activities but able to look after own affairs without assistance. NIHSS improved from 8 to 3. Patient discharged on hospital day 8 to home with outpatient physical therapy and speech therapy referrals. Chronic transfusion therapy restarted to maintain HbS below 30%. Follow-up with neurology in 2 weeks and hematology in 1 week.
+DISCHARGE DIAGNOSES: (1) Acute ischemic stroke, left MCA territory, with residual right hemiparesis and mild dysarthria; stroke symptoms present and not fully resolved at discharge; mRS 2. (2) No concurrent vaso-occlusive pain crisis — no pain reported during admission.</t>
+        </is>
+      </c>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>7/15/94</t>
+        </is>
+      </c>
+      <c r="M27" s="10" t="inlineStr">
+        <is>
+          <t>10/1/94</t>
+        </is>
+      </c>
+      <c r="N27" s="10" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr"/>
+      <c r="Q27" s="12" t="inlineStr"/>
+      <c r="R27" s="12" t="inlineStr"/>
+      <c r="S27" s="12" t="inlineStr"/>
+      <c r="T27" s="12" t="inlineStr"/>
+      <c r="U27" s="12" t="inlineStr"/>
+      <c r="V27" s="12" t="inlineStr"/>
+      <c r="W27" s="12" t="inlineStr"/>
+      <c r="X27" s="12" t="inlineStr"/>
+      <c r="Y27" s="12" t="inlineStr"/>
+      <c r="Z27" s="12" t="inlineStr"/>
+      <c r="AA27" s="12" t="inlineStr"/>
+      <c r="AB27" s="12" t="inlineStr"/>
+      <c r="AC27" s="12" t="inlineStr"/>
+      <c r="AD27" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AE27" s="12" t="inlineStr"/>
+      <c r="AF27" s="12" t="inlineStr"/>
+      <c r="AG27" s="12" t="inlineStr"/>
+      <c r="AH27" s="12" t="inlineStr"/>
+      <c r="AI27" s="12" t="inlineStr"/>
+      <c r="AJ27" s="12" t="inlineStr"/>
+      <c r="AK27" s="12" t="inlineStr"/>
+      <c r="AL27" s="12" t="inlineStr"/>
+      <c r="AM27" s="12" t="inlineStr"/>
+      <c r="AN27" s="12" t="inlineStr"/>
+      <c r="AO27" s="12" t="inlineStr"/>
+      <c r="AP27" s="12" t="inlineStr"/>
+      <c r="AQ27" s="12" t="inlineStr"/>
+      <c r="AR27" s="12" t="inlineStr"/>
+      <c r="AS27" s="12" t="inlineStr"/>
+      <c r="AT27" s="12" t="inlineStr"/>
+      <c r="AU27" s="12" t="inlineStr"/>
+      <c r="AV27" s="12" t="inlineStr"/>
+      <c r="AW27" s="12" t="inlineStr"/>
+      <c r="AX27" s="12" t="inlineStr"/>
+      <c r="AY27" s="12" t="inlineStr"/>
+      <c r="AZ27" s="12" t="inlineStr"/>
+      <c r="BA27" s="12" t="inlineStr"/>
+      <c r="BB27" s="12" t="inlineStr"/>
+      <c r="BC27" s="12" t="inlineStr"/>
+      <c r="BD27" s="12" t="inlineStr"/>
+      <c r="BE27" s="12" t="inlineStr"/>
+      <c r="BF27" s="12" t="inlineStr"/>
+      <c r="BG27" s="12" t="inlineStr"/>
+      <c r="BH27" s="12" t="inlineStr"/>
+      <c r="BI27" s="12" t="inlineStr"/>
+      <c r="BJ27" s="12" t="inlineStr"/>
+      <c r="BK27" s="12" t="inlineStr"/>
+      <c r="BL27" s="12" t="inlineStr"/>
+      <c r="BM27" s="12" t="inlineStr"/>
+      <c r="BN27" s="12" t="inlineStr"/>
+      <c r="BO27" s="12" t="inlineStr"/>
+      <c r="BP27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28" ht="200" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_011</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>12/20/25</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Leg Pain</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 8-year-old male with sickle cell disease (HbSS), history of functional asplenia (Howell-Jolly bodies on smear, no prior splenectomy), presents to the pediatric emergency department with high fever, rigors, and lethargy since this morning. His mother reports his temperature at home was 39.4 degrees Celsius (102.9 degrees Fahrenheit). He has been less active and not eating. He also complains of mild bilateral leg pain rated 4 out of 10. He denies cough, shortness of breath, chest pain, headache, abdominal pain, or urinary symptoms. He is up to date on pneumococcal vaccination (PCV13 and PPSV23). He takes daily prophylactic penicillin VK. No recent hospitalizations.
+OBJECTIVE: Temperature 39.6 degrees Celsius (103.3 degrees Fahrenheit), heart rate 142 bpm, blood pressure 88/52 mmHg (age-appropriate threshold for hypotension in 8-year-old: SBP &lt; 70 + [2 x age] = &lt; 86 mmHg), respiratory rate 28 breaths/min, SpO2 96% on room air. Weight: 24 kg. General: Lethargic-appearing child, arousable, responds to voice. HEENT: Scleral icterus. Mucous membranes dry. Lungs: Clear to auscultation bilaterally, no wheezes or crackles. Cardiovascular: Tachycardic, regular rhythm, grade II/VI systolic flow murmur. Capillary refill: 3 seconds centrally. Abdomen: Soft, mildly tender diffusely, no organomegaly (functionally asplenic). Extremities: Bilateral tibial tenderness, no swelling, no calf tenderness, no skin lesions, no leg ulcers. Neurological: Lethargic but oriented when stimulated, GCS 14 (E3 V5 M6), no focal deficits, no neck stiffness.
+LABS: Hemoglobin 7.2 g/dL (baseline 7.8 g/dL), WBC 22.4 x 10^3/uL with 12% bands and toxic granulations, platelets 156 x 10^3/uL. Reticulocyte count 10.2%. Serum creatinine 0.5 mg/dL (baseline 0.4 mg/dL, 1.25x baseline). LDH 320 U/L, total bilirubin 2.6 mg/dL. Lactate 3.2 mmol/L (elevated). Procalcitonin 4.8 ng/mL. CRP 142 mg/L. Urinalysis: No evidence of UTI. Chest X-ray: Clear lungs bilaterally, no infiltrates, no pleural effusion — no evidence of acute chest syndrome. Blood cultures: Two sets drawn from peripheral sites.
+HOSPITAL COURSE: Given the combination of high fever, tachycardia, borderline hypotension, lethargy, and elevated lactate in a functionally asplenic child with SCD, the clinical picture was concerning for sepsis. Empiric antibiotics initiated within 30 minutes of arrival: ceftriaxone 100 mg/kg IV (2.4 g) and vancomycin 15 mg/kg IV. Normal saline bolus 20 mL/kg (480 mL) administered with improvement in blood pressure to 96/60 mmHg and heart rate to 118 bpm. A second 10 mL/kg bolus was given. Patient did NOT require vasopressors, mechanical ventilation, or any other life-support interventions. Patient admitted to the medical floor (not ICU).
+On hospital day 1, blood cultures (both sets) grew Streptococcus pneumoniae, serotype 19A, susceptible to ceftriaxone. Vancomycin discontinued. Lactate normalized to 1.4 mmol/L by day 2. Mental status returned to baseline by day 1. Fever resolved by day 2. Mild leg pain managed with oral ibuprofen and resolved by day 2. Creatinine remained stable at 0.5 mg/dL. No respiratory distress, no new infiltrates — ACS ruled out. No neurological complications. No arrhythmias.
+DISCHARGE: Patient discharged on hospital day 4 in good condition, completing IV antibiotics transitioned to oral amoxicillin for a 10-day total course. Follow-up in 48 hours.
+DISCHARGE DIAGNOSES: (1) Sepsis secondary to Streptococcus pneumoniae bacteremia with organ dysfunction (elevated lactate, tachycardia, borderline hypotension, lethargy); blood culture positive; treated with antibiotics and fluid resuscitation; no vasopressors or life-support required; not life-threatening. (2) Acute sickle cell pain episode, mild, managed with oral analgesics during hospitalization; admitted to medical floor; no co-complications. (3) Fever, temperature 39.6 degrees Celsius.</t>
+        </is>
+      </c>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t>4/8/17</t>
+        </is>
+      </c>
+      <c r="M28" s="10" t="inlineStr">
+        <is>
+          <t>4/12/17</t>
+        </is>
+      </c>
+      <c r="N28" s="10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P28" s="12" t="inlineStr"/>
+      <c r="Q28" s="12" t="inlineStr"/>
+      <c r="R28" s="12" t="inlineStr"/>
+      <c r="S28" s="12" t="inlineStr"/>
+      <c r="T28" s="12" t="inlineStr"/>
+      <c r="U28" s="12" t="inlineStr"/>
+      <c r="V28" s="12" t="inlineStr"/>
+      <c r="W28" s="12" t="inlineStr"/>
+      <c r="X28" s="12" t="inlineStr"/>
+      <c r="Y28" s="12" t="inlineStr"/>
+      <c r="Z28" s="12" t="inlineStr"/>
+      <c r="AA28" s="12" t="inlineStr"/>
+      <c r="AB28" s="12" t="inlineStr"/>
+      <c r="AC28" s="12" t="inlineStr"/>
+      <c r="AD28" s="12" t="inlineStr"/>
+      <c r="AE28" s="12" t="inlineStr"/>
+      <c r="AF28" s="12" t="inlineStr"/>
+      <c r="AG28" s="12" t="inlineStr"/>
+      <c r="AH28" s="12" t="inlineStr"/>
+      <c r="AI28" s="12" t="inlineStr"/>
+      <c r="AJ28" s="12" t="inlineStr"/>
+      <c r="AK28" s="12" t="inlineStr"/>
+      <c r="AL28" s="12" t="inlineStr"/>
+      <c r="AM28" s="12" t="inlineStr"/>
+      <c r="AN28" s="12" t="inlineStr"/>
+      <c r="AO28" s="12" t="inlineStr"/>
+      <c r="AP28" s="12" t="inlineStr"/>
+      <c r="AQ28" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AR28" s="12" t="inlineStr"/>
+      <c r="AS28" s="12" t="inlineStr"/>
+      <c r="AT28" s="12" t="inlineStr"/>
+      <c r="AU28" s="12" t="inlineStr"/>
+      <c r="AV28" s="12" t="inlineStr"/>
+      <c r="AW28" s="12" t="inlineStr"/>
+      <c r="AX28" s="12" t="inlineStr"/>
+      <c r="AY28" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AZ28" s="13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="BA28" s="12" t="inlineStr"/>
+      <c r="BB28" s="12" t="inlineStr"/>
+      <c r="BC28" s="12" t="inlineStr"/>
+      <c r="BD28" s="12" t="inlineStr"/>
+      <c r="BE28" s="12" t="inlineStr"/>
+      <c r="BF28" s="12" t="inlineStr"/>
+      <c r="BG28" s="12" t="inlineStr"/>
+      <c r="BH28" s="12" t="inlineStr"/>
+      <c r="BI28" s="12" t="inlineStr"/>
+      <c r="BJ28" s="12" t="inlineStr"/>
+      <c r="BK28" s="12" t="inlineStr"/>
+      <c r="BL28" s="12" t="inlineStr"/>
+      <c r="BM28" s="12" t="inlineStr"/>
+      <c r="BN28" s="12" t="inlineStr"/>
+      <c r="BO28" s="12" t="inlineStr"/>
+      <c r="BP28" s="12" t="inlineStr"/>
+    </row>
+    <row r="29" ht="200" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>SYNTH_012</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>2/14/26</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>ER</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>Leg Pain</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>SUBJECTIVE: 27-year-old female with sickle cell disease (HbSS) presents to the emergency department with bilateral lower extremity pain rated 6 out of 10 for the past 12 hours. She reports feeling warm but has not checked her temperature. She denies cough, shortness of breath, chest pain, abdominal pain, headache, vision changes, leg swelling, or urinary symptoms. She reports mild right calf discomfort but attributes it to her pain crisis. She has been feeling mildly sad over the past few weeks since a relationship breakup but states she is coping well. No suicidal ideation. She is eating and sleeping adequately. No history of prior DVT, PE, or stroke.
+OBJECTIVE: Temperature 37.9 degrees Celsius (100.2 degrees Fahrenheit), heart rate 90 bpm, blood pressure 120/74 mmHg, respiratory rate 18 breaths/min, SpO2 97% on room air. General: Alert, oriented, mildly uncomfortable. HEENT: Mild scleral icterus. Lungs: Clear to auscultation bilaterally, no wheezes, no crackles. Cardiovascular: Regular rate and rhythm, no murmurs. Abdomen: Soft, non-tender, no hepatosplenomegaly. Right lower extremity: Mild calf tenderness to deep palpation, no swelling, no erythema, no warmth, no pitting edema, negative Homans sign. Left lower extremity: Unremarkable. No leg ulcers bilaterally. Neurological: Alert and oriented x4, cranial nerves II-XII intact, no focal deficits. Psychiatric: Mildly low affect but appropriate. PHQ-2 screening: score 2 out of 6 (below threshold for full PHQ-9 assessment).
+LABS: Hemoglobin 8.0 g/dL (baseline 8.4 g/dL), WBC 10.1 x 10^3/uL, platelets 280 x 10^3/uL. Serum creatinine 0.84 mg/dL (baseline 0.6 mg/dL, representing 1.40 times baseline — note: this is below the 1.5x threshold for AKI Grade 1). D-dimer 0.8 mg/L (mildly elevated). LDH 310 U/L, total bilirubin 2.9 mg/dL.
+IMAGING: Given mild right calf tenderness and elevated D-dimer, bilateral lower extremity venous Doppler ultrasound was obtained: Normal compressibility of all deep veins bilaterally. No evidence of deep vein thrombosis. Chest X-ray: A small area of subsegmental atelectasis in the right lower lobe, likely positional. No lobar or segmental consolidation. No infiltrate meeting criteria for acute chest syndrome. No pleural effusion.
+ASSESSMENT: (1) Acute sickle cell vaso-occlusive pain episode. (2) Temperature 37.9 degrees Celsius — below the 38.0 degrees Celsius threshold for SCOGS fever grading; does not qualify as fever. (3) Creatinine 1.40 times baseline — below the 1.5 times baseline threshold for SCOGS AKI Grade 1; does not qualify as acute kidney injury. (4) Right lower lobe subsegmental atelectasis — does NOT meet radiographic criteria for acute chest syndrome (requires new lobar or segmental infiltrate, not atelectasis). (5) Normal bilateral lower extremity venous Doppler — no DVT. (6) PHQ-2 score 2 — below the screening threshold; formal PHQ-9 not indicated; does not meet criteria for SCOGS depression grading.
+PLAN: IV normal saline 1 liter bolus. IV morphine 4 mg with reassessment. After 3 hours in the ED, pain improved to 3 out of 10. Patient does not require admission. Discharged home with oral analgesics and hydration instructions. Instructed to return if temperature reaches 38.0 degrees Celsius or above, or if symptoms worsen. Follow-up with hematology clinic in 48 hours.
+DISCHARGE DIAGNOSES: (1) Acute sickle cell pain episode, managed in ED, not admitted.</t>
+        </is>
+      </c>
+      <c r="L29" s="10" t="inlineStr">
+        <is>
+          <t>9/3/98</t>
+        </is>
+      </c>
+      <c r="M29" s="10" t="inlineStr">
+        <is>
+          <t>12/1/98</t>
+        </is>
+      </c>
+      <c r="N29" s="10" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>Black or African American</t>
+        </is>
+      </c>
+      <c r="P29" s="12" t="inlineStr"/>
+      <c r="Q29" s="12" t="inlineStr"/>
+      <c r="R29" s="12" t="inlineStr"/>
+      <c r="S29" s="12" t="inlineStr"/>
+      <c r="T29" s="12" t="inlineStr"/>
+      <c r="U29" s="12" t="inlineStr"/>
+      <c r="V29" s="12" t="inlineStr"/>
+      <c r="W29" s="12" t="inlineStr"/>
+      <c r="X29" s="12" t="inlineStr"/>
+      <c r="Y29" s="12" t="inlineStr"/>
+      <c r="Z29" s="12" t="inlineStr"/>
+      <c r="AA29" s="12" t="inlineStr"/>
+      <c r="AB29" s="12" t="inlineStr"/>
+      <c r="AC29" s="12" t="inlineStr"/>
+      <c r="AD29" s="12" t="inlineStr"/>
+      <c r="AE29" s="12" t="inlineStr"/>
+      <c r="AF29" s="12" t="inlineStr"/>
+      <c r="AG29" s="12" t="inlineStr"/>
+      <c r="AH29" s="12" t="inlineStr"/>
+      <c r="AI29" s="12" t="inlineStr"/>
+      <c r="AJ29" s="12" t="inlineStr"/>
+      <c r="AK29" s="12" t="inlineStr"/>
+      <c r="AL29" s="12" t="inlineStr"/>
+      <c r="AM29" s="12" t="inlineStr"/>
+      <c r="AN29" s="12" t="inlineStr"/>
+      <c r="AO29" s="12" t="inlineStr"/>
+      <c r="AP29" s="12" t="inlineStr"/>
+      <c r="AQ29" s="13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AR29" s="12" t="inlineStr"/>
+      <c r="AS29" s="12" t="inlineStr"/>
+      <c r="AT29" s="12" t="inlineStr"/>
+      <c r="AU29" s="12" t="inlineStr"/>
+      <c r="AV29" s="12" t="inlineStr"/>
+      <c r="AW29" s="12" t="inlineStr"/>
+      <c r="AX29" s="12" t="inlineStr"/>
+      <c r="AY29" s="12" t="inlineStr"/>
+      <c r="AZ29" s="12" t="inlineStr"/>
+      <c r="BA29" s="12" t="inlineStr"/>
+      <c r="BB29" s="12" t="inlineStr"/>
+      <c r="BC29" s="12" t="inlineStr"/>
+      <c r="BD29" s="12" t="inlineStr"/>
+      <c r="BE29" s="12" t="inlineStr"/>
+      <c r="BF29" s="12" t="inlineStr"/>
+      <c r="BG29" s="12" t="inlineStr"/>
+      <c r="BH29" s="12" t="inlineStr"/>
+      <c r="BI29" s="12" t="inlineStr"/>
+      <c r="BJ29" s="12" t="inlineStr"/>
+      <c r="BK29" s="12" t="inlineStr"/>
+      <c r="BL29" s="12" t="inlineStr"/>
+      <c r="BM29" s="12" t="inlineStr"/>
+      <c r="BN29" s="12" t="inlineStr"/>
+      <c r="BO29" s="12" t="inlineStr"/>
+      <c r="BP29" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A17:BP25"/>
+  <autoFilter ref="A17:BP29"/>
   <mergeCells count="14">
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A1:G1"/>
@@ -2366,7 +2943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3659,86 +4236,667 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="22" t="inlineStr">
+    <row r="56" ht="55" customHeight="1">
+      <c r="A56" s="15" t="inlineStr"/>
+      <c r="B56" s="15" t="inlineStr"/>
+      <c r="C56" s="15" t="inlineStr"/>
+      <c r="D56" s="15" t="inlineStr"/>
+      <c r="E56" s="15" t="inlineStr"/>
+      <c r="F56" s="15" t="inlineStr"/>
+      <c r="G56" s="15" t="inlineStr"/>
+    </row>
+    <row r="57" ht="55" customHeight="1">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_009
+(Note 9)</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>Acute Chest Syndrome</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="D57" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>fio2_pct = 28%
+resp_support = nasal_cannula
+transfusion_type = simple
+acs_other_support = false
+life_support = false</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>(fio2 &lt; 50 AND no high_flow AND no exchange) AND (simple OR O2 OR other_support) → Grade 2</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="inlineStr">
+        <is>
+          <t>"nasal cannula at 2 L/min (FiO2 approximately 28%)"; "2 units of packed red blood cells"</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_009
+(Note 9)</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C58" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E58" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = inpatient
+pain_co_complication = false</t>
+        </is>
+      </c>
+      <c r="F58" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ inpatient AND NOT co_complication → Grade 3</t>
+        </is>
+      </c>
+      <c r="G58" s="15" t="inlineStr">
+        <is>
+          <t>"Patient admitted to the medical floor"; "without co-complications"</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="55" customHeight="1">
+      <c r="A59" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_009
+(Note 9)</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C59" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D59" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E59" s="15" t="inlineStr">
+        <is>
+          <t>temperature = 39.0 °C</t>
+        </is>
+      </c>
+      <c r="F59" s="15" t="inlineStr">
+        <is>
+          <t>temp ≥ 38.5 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G59" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 39.0 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="55" customHeight="1">
+      <c r="A60" s="15" t="inlineStr"/>
+      <c r="B60" s="15" t="inlineStr"/>
+      <c r="C60" s="15" t="inlineStr"/>
+      <c r="D60" s="15" t="inlineStr"/>
+      <c r="E60" s="15" t="inlineStr"/>
+      <c r="F60" s="15" t="inlineStr"/>
+      <c r="G60" s="15" t="inlineStr"/>
+    </row>
+    <row r="61" ht="55" customHeight="1">
+      <c r="A61" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_010
+(Note 10)</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
+          <t>Stroke</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>#15</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E61" s="15" t="inlineStr">
+        <is>
+          <t>stroke_symptoms = true
+stroke_symptoms_resolved = false
+mrs = 2</t>
+        </is>
+      </c>
+      <c r="F61" s="15" t="inlineStr">
+        <is>
+          <t>stroke_symptoms AND NOT resolved AND 1 &lt;= mrs &lt;= 3 → Grade 3</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr">
+        <is>
+          <t>"right-sided weakness and slurred speech"; "stroke symptoms present and not fully resolved... mRS 2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="55" customHeight="1">
+      <c r="A62" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_010
+(Note 10)</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E62" s="15" t="inlineStr">
+        <is>
+          <t>No pain reported</t>
+        </is>
+      </c>
+      <c r="F62" s="15" t="inlineStr">
+        <is>
+          <t>No vaso-occlusive pain crisis → absent</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>"No concurrent vaso-occlusive pain crisis — no pain reported"</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="55" customHeight="1">
+      <c r="A63" s="15" t="inlineStr"/>
+      <c r="B63" s="15" t="inlineStr"/>
+      <c r="C63" s="15" t="inlineStr"/>
+      <c r="D63" s="15" t="inlineStr"/>
+      <c r="E63" s="15" t="inlineStr"/>
+      <c r="F63" s="15" t="inlineStr"/>
+      <c r="G63" s="15" t="inlineStr"/>
+    </row>
+    <row r="64" ht="55" customHeight="1">
+      <c r="A64" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_011
+(Note 11)</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>Sepsis</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>#37</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E64" s="15" t="inlineStr">
+        <is>
+          <t>blood_culture_positive = true
+organ_dysfunction = true
+treated = true
+life_threatening_sepsis = false
+life_support = false</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>blood_culture_positive AND (organ_dysfunction OR treated) → Grade 3</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>"blood cultures... grew Streptococcus pneumoniae"; "elevated lactate"</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="55" customHeight="1">
+      <c r="A65" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_011
+(Note 11)</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D65" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E65" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = inpatient
+pain_co_complication = false</t>
+        </is>
+      </c>
+      <c r="F65" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ inpatient AND NOT co_complication → Grade 3</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>"Patient admitted to the medical floor"; "no co-complications"</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="55" customHeight="1">
+      <c r="A66" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_011
+(Note 11)</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E66" s="15" t="inlineStr">
+        <is>
+          <t>temperature = 39.6 °C</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>temp ≥ 38.5 → Grade 2</t>
+        </is>
+      </c>
+      <c r="G66" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 39.6 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="55" customHeight="1">
+      <c r="A67" s="15" t="inlineStr"/>
+      <c r="B67" s="15" t="inlineStr"/>
+      <c r="C67" s="15" t="inlineStr"/>
+      <c r="D67" s="15" t="inlineStr"/>
+      <c r="E67" s="15" t="inlineStr"/>
+      <c r="F67" s="15" t="inlineStr"/>
+      <c r="G67" s="15" t="inlineStr"/>
+    </row>
+    <row r="68" ht="55" customHeight="1">
+      <c r="A68" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_012
+(Note 12)</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="inlineStr">
+        <is>
+          <t>Acute Sickle Cell Pain Episode</t>
+        </is>
+      </c>
+      <c r="C68" s="15" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E68" s="15" t="inlineStr">
+        <is>
+          <t>care_setting = ed_treat_release
+pain_co_complication = false</t>
+        </is>
+      </c>
+      <c r="F68" s="15" t="inlineStr">
+        <is>
+          <t>care_setting ≥ clinic AND &lt; inpatient → Grade 2</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="inlineStr">
+        <is>
+          <t>"After 3 hours in the ED... Patient does not require admission. Discharged home"</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="55" customHeight="1">
+      <c r="A69" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_012
+(Note 12)</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Fever</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>#36</t>
+        </is>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E69" s="15" t="inlineStr">
+        <is>
+          <t>temperature = 37.9 °C</t>
+        </is>
+      </c>
+      <c r="F69" s="15" t="inlineStr">
+        <is>
+          <t>temp &lt; 38.0 → absent (0.1° below threshold)</t>
+        </is>
+      </c>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>"Temperature 37.9 degrees Celsius"</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="55" customHeight="1">
+      <c r="A70" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_012
+(Note 12)</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
+        <is>
+          <t>Acute Kidney Injury</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>#19</t>
+        </is>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E70" s="15" t="inlineStr">
+        <is>
+          <t>creatinine_x_baseline = 1.40</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr">
+        <is>
+          <t>creat_x_base &lt; 1.5 → absent (0.1x below threshold)</t>
+        </is>
+      </c>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>"creatinine... representing 1.40 times baseline"</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="55" customHeight="1">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_012
+(Note 12)</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>Acute Chest Syndrome</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E71" s="15" t="inlineStr">
+        <is>
+          <t>atelectasis</t>
+        </is>
+      </c>
+      <c r="F71" s="15" t="inlineStr">
+        <is>
+          <t>No lobar/segmental infiltrate → absent</t>
+        </is>
+      </c>
+      <c r="G71" s="15" t="inlineStr">
+        <is>
+          <t>"subsegmental atelectasis... No lobar or segmental consolidation"</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="55" customHeight="1">
+      <c r="A72" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_012
+(Note 12)</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>Deep Vein Thrombosis</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>#02</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>Negative Doppler</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>Requires positive imaging → absent</t>
+        </is>
+      </c>
+      <c r="G72" s="15" t="inlineStr">
+        <is>
+          <t>"Normal compressibility of all deep veins bilaterally"</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="55" customHeight="1">
+      <c r="A73" s="15" t="inlineStr">
+        <is>
+          <t>SYNTH_012
+(Note 12)</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>Depression</t>
+        </is>
+      </c>
+      <c r="C73" s="15" t="inlineStr">
+        <is>
+          <t>#47</t>
+        </is>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="E73" s="15" t="inlineStr">
+        <is>
+          <t>PHQ-2 = 2</t>
+        </is>
+      </c>
+      <c r="F73" s="15" t="inlineStr">
+        <is>
+          <t>PHQ-9 ≥ 5 required → absent</t>
+        </is>
+      </c>
+      <c r="G73" s="15" t="inlineStr">
+        <is>
+          <t>"PHQ-2 score 2 — below the screening threshold"</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="inlineStr">
         <is>
           <t>Grade Legend:</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="23" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="23" t="inlineStr">
         <is>
           <t>Grade 1 — Mild</t>
         </is>
       </c>
-      <c r="B59" s="6" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="24" t="inlineStr">
+      <c r="B77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="24" t="inlineStr">
         <is>
           <t>Grade 2 — Moderate</t>
         </is>
       </c>
-      <c r="B60" s="6" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="25" t="inlineStr">
+      <c r="B78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="25" t="inlineStr">
         <is>
           <t>Grade 3 — Severe</t>
         </is>
       </c>
-      <c r="B61" s="6" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="26" t="inlineStr">
+      <c r="B79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="26" t="inlineStr">
         <is>
           <t>Grade 4 — Life-Threatening</t>
         </is>
       </c>
-      <c r="B62" s="6" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="27" t="inlineStr">
+      <c r="B80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="27" t="inlineStr">
         <is>
           <t>Grade 5 — Fatal</t>
         </is>
       </c>
-      <c r="B63" s="6" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="28" t="inlineStr">
+      <c r="B81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="28" t="inlineStr">
         <is>
           <t>Absent — Outcome not present</t>
         </is>
       </c>
-      <c r="B64" s="6" t="n"/>
+      <c r="B82" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="24">
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A82:B82"/>
     <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A60:B60"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A79:B79"/>
     <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A61:B61"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A78:B78"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A80:B80"/>
     <mergeCell ref="A11:G11"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A62:B62"/>
     <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A81:B81"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A77:B77"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>